<commit_message>
Profile all workloads on RTX 4090 (nsys and timing) and add 4090 sheet
Rebuilds every workload for sm_89 with CUDA 12.5 (this host's driver
supports up to 12.5) into rtx4090/ and reruns the nsys traces, the
llama2c GPU-filling sweep and the loom_msa benchmark with the RTX 3090
runs' arguments. The spreadsheet gets an "RTX 4090" summary sheet read
from rtx4090/; the 3090 sheet is unchanged apart from its title, and its
notes are now computed from the reports instead of hard-coded.

ncu cannot read performance counters here without admin rights, so the
4090 kernel-time rows read "pending" until profile_ncu_all.sh (new) is
run with sudo; rerunning build_spreadsheet.py then fills them in.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/cuda_performance.xlsx
+++ b/results/cuda_performance.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ncu metrics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RTX 3090" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RTX 4090" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="ncu metrics (RTX 3090)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ncu metrics (RTX 4090)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -139,10 +141,14 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,14 +535,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CUDA performance results (latest runs)</t>
+          <t>CUDA performance results (latest runs): RTX 3090</t>
         </is>
       </c>
     </row>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GPU: NVIDIA GeForce RTX 3090 (sm_86, 24 GB). Times in microseconds (lower is better). Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so ncu kernel times barely change with launch mode; the CUDA Graph benefit (launch overhead) shows in end-to-end rows.</t>
+          <t>GPU: NVIDIA GeForce RTX 3090 (sm_86, 24 GB), binaries built with CUDA 13.3 GPU (outputs in rtx3090/). Times in microseconds (lower is better). Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so ncu kernel times barely change with launch mode; the CUDA Graph benefit (launch overhead) shows in end-to-end rows.</t>
         </is>
       </c>
     </row>
@@ -1347,6 +1353,813 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CUDA performance results (latest runs): RTX 4090</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GPU: NVIDIA GeForce RTX 4090 (sm_89, 24 GB), binaries built with CUDA 12.5 GPU (outputs in rtx4090/). Times in microseconds (lower is better). Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so ncu kernel times barely change with launch mode; the CUDA Graph benefit (launch overhead) shows in end-to-end rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Workload</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Kernel / stage</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Problem size</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>CUDA Graph</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Direct launch (no graph)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Graph speedup
+(Direct / Graph)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Time (us)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>ncu-rep</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>nsys sqlite</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Time (us)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>ncu-rep</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>nsys sqlite</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>llama2c (coalesced matmul)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>matmul_coalesced_kernel</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>batch=1024, dim=16384, rows=8192</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>nsys-node-graph-20261015-091930.sqlite</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>nsys-node-direct-20261015-091935.sqlite</t>
+        </is>
+      </c>
+      <c r="L6" s="10">
+        <f>IF(AND(ISNUMBER(F6),ISNUMBER(I6)),I6/F6,"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Largest kernel. It is a matrix-vector product, so its time does not grow with batch; the three kernels run concurrently on separate streams, so their times overlap. </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>llama2c (coalesced matmul)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (rmsnorm + softmax + matmul iteration)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>batch=1024, dim=16384, rows=8192</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Iteration time (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>962.42</v>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>nsys-node-graph-20261015-091930.sqlite</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>963.302</v>
+      </c>
+      <c r="J7" s="12" t="n"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>nsys-node-direct-20261015-091935.sqlite</t>
+        </is>
+      </c>
+      <c r="L7" s="10">
+        <f>IF(AND(ISNUMBER(F7),ISNUMBER(I7)),I7/F7,"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="5" t="inlineStr">
+        <is>
+          <t>Mean of 3 interleaved trials from the GPU-filling sweep; no per-iteration copies. The nsys traces rerun this configuration (963.0 / 962.1 us per iteration).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>loom_msa (multi-sensor attention)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>fuse_attention_kernel</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>25,000 queries x 250,000 context</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>nsys-msa_optimized_large-20261015-091307.sqlite</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="10">
+        <f>IF(AND(ISNUMBER(F9),ISNUMBER(I9)),I9/F9,"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style). </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>loom_msa (multi-sensor attention)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (graph replay)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>25,000 queries x 250,000 context</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Replay time (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>3835.57</v>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>nsys-msa_optimized_large-20261015-091307.sqlite</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="10">
+        <f>IF(AND(ISNUMBER(F10),ISNUMBER(I10)),I10/F10,"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="5" t="inlineStr">
+        <is>
+          <t>benchmark.py: median of 5 runs, random inputs. Includes H2D input and D2H output copies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>pagerank (GAPBS)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>pagerank_update (one iteration)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>nsys-20261015-091708.sqlite</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="10">
+        <f>IF(AND(ISNUMBER(F12),ISNUMBER(I12)),I12/F12,"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pull gather of precomputed contributions. Full-graph iterations only; the first iteration runs as 8 upload-overlapped chunks. </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>pagerank (GAPBS)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (graph replay: H2D + 20 iterations)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Replay time (nsys)</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>5754.945</v>
+      </c>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>nsys-20261015-091708.sqlite</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="10">
+        <f>IF(AND(ISNUMBER(F13),ISNUMBER(I13)),I13/F13,"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Median span of the 1693 replays with transfers in the nsys node trace. The CSR graph is uploaded from pinned memory in 8 chunks overlapped with the first iteration. A separate uninstrumented run of the binary (profiles/bench-20261015-091815.txt): 5.714 ms with transfers, 2.651 ms compute only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny anomaly</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>mse_partial_kernel</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>64M elements</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="10">
+        <f>IF(AND(ISNUMBER(F15),ISNUMBER(I15)),I15/F15,"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny anomaly</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (graph replay: H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>64M elements</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Replay time (nsys)</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>13698.465</v>
+      </c>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="10">
+        <f>IF(AND(ISNUMBER(F16),ISNUMBER(I16)),I16/F16,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>kws_postprocess_kernel</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 4M rows</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="10">
+        <f>IF(AND(ISNUMBER(F18),ISNUMBER(I18)),I18/F18,"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only kernel in the application. </t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (graph replay: H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 4M rows</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Replay time (nsys)</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>11226.082</v>
+      </c>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="10">
+        <f>IF(AND(ISNUMBER(F19),ISNUMBER(I19)),I19/F19,"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>vww_preprocess_kernel</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu)</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="10">
+        <f>IF(AND(ISNUMBER(F21),ISNUMBER(I21)),I21/F21,"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only kernel in the application. </t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (graph replay: H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Replay time (nsys)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>21789.123</v>
+      </c>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>n/a (graph-only harness)</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n"/>
+      <c r="K22" s="12" t="n"/>
+      <c r="L22" s="10">
+        <f>IF(AND(ISNUMBER(F22),ISNUMBER(I22)),I22/F22,"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1368,84 +2181,84 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>ncu report</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Launch #</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Kernel</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>SM throughput %</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Memory throughput %</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>DRAM throughput %</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Achieved occupancy %</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Theoretical occupancy %</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>Registers / thread</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="15" t="inlineStr">
         <is>
           <t>Grid</t>
         </is>
       </c>
-      <c r="L1" s="14" t="inlineStr">
+      <c r="L1" s="15" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="M1" s="14" t="inlineStr">
+      <c r="M1" s="15" t="inlineStr">
         <is>
           <t>Waves / SM</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="15" t="inlineStr">
         <is>
           <t>DRAM read</t>
         </is>
       </c>
-      <c r="O1" s="14" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>DRAM write</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1496,7 +2309,7 @@
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1547,7 +2360,7 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1598,7 +2411,7 @@
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1649,7 +2462,7 @@
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1700,7 +2513,7 @@
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1751,7 +2564,7 @@
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1802,7 +2615,7 @@
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1853,7 +2666,7 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -1904,7 +2717,7 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -1955,7 +2768,7 @@
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2006,7 +2819,7 @@
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2057,7 +2870,7 @@
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2108,7 +2921,7 @@
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2159,7 +2972,7 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2210,7 +3023,7 @@
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2261,7 +3074,7 @@
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2312,7 +3125,7 @@
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2363,7 +3176,7 @@
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -2414,7 +3227,7 @@
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -2465,7 +3278,7 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -2516,7 +3329,7 @@
       <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -2567,7 +3380,7 @@
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2626,7 +3439,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2685,7 +3498,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2744,7 +3557,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2803,7 +3616,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2862,7 +3675,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2921,7 +3734,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -2980,7 +3793,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3039,7 +3852,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3098,7 +3911,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3157,7 +3970,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3216,7 +4029,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3275,7 +4088,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3334,7 +4147,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3393,7 +4206,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3452,7 +4265,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3511,7 +4324,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3570,7 +4383,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3629,7 +4442,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="inlineStr">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3688,7 +4501,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="15" t="inlineStr">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3747,7 +4560,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3806,7 +4619,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3865,7 +4678,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3924,7 +4737,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="15" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3983,7 +4796,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="15" t="inlineStr">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4042,7 +4855,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="15" t="inlineStr">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4101,7 +4914,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="15" t="inlineStr">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4160,7 +4973,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4219,7 +5032,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="15" t="inlineStr">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t>ncu-anomaly_mse-20261007-144943.ncu-rep</t>
         </is>
@@ -4278,7 +5091,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t>ncu-anomaly_mse-20261007-144943.ncu-rep</t>
         </is>
@@ -4337,7 +5150,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="15" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t>ncu-kws_postprocess-20261007-144950.ncu-rep</t>
         </is>
@@ -4396,7 +5209,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="15" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>ncu-vww_preprocess-20261007-144958.ncu-rep</t>
         </is>
@@ -4513,4 +5326,119 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>ncu report</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Launch #</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Kernel</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>SM throughput %</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Memory throughput %</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>DRAM throughput %</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>Achieved occupancy %</t>
+        </is>
+      </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Theoretical occupancy %</t>
+        </is>
+      </c>
+      <c r="J1" s="15" t="inlineStr">
+        <is>
+          <t>Registers / thread</t>
+        </is>
+      </c>
+      <c r="K1" s="15" t="inlineStr">
+        <is>
+          <t>Grid</t>
+        </is>
+      </c>
+      <c r="L1" s="15" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="M1" s="15" t="inlineStr">
+        <is>
+          <t>Waves / SM</t>
+        </is>
+      </c>
+      <c r="N1" s="15" t="inlineStr">
+        <is>
+          <t>DRAM read</t>
+        </is>
+      </c>
+      <c r="O1" s="15" t="inlineStr">
+        <is>
+          <t>DRAM write</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compare RTX 4090 against RTX 3090: predicted and measured speedup
The RTX 4090 sheet replaces its Direct / Graph speedup column with two
columns against the RTX 3090. Predicted speedup is a bottleneck model
from the 3090 ncu reports' per-unit throughput and both GPUs' specs.
Measured speedup divides the 3090's CUDA Graph time by the 4090's.
The method is explained under the table and in the README.
</commit_message>
<xml_diff>
--- a/results/cuda_performance.xlsx
+++ b/results/cuda_performance.xlsx
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -142,6 +142,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -223,6 +227,76 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>build_spreadsheet.py</author>
+  </authors>
+  <commentList>
+    <comment ref="L6" authorId="0" shapeId="0">
+      <text>
+        <t>DRAM-bound (DRAM 94% busy; SM 5%, L1/L2 94%): data rate 21 / 18.98 Gbps = 1.11x.</t>
+      </text>
+    </comment>
+    <comment ref="L7" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels overlap (their summed ncu time is 105% of this time), so all of it scales with the kernels' 1.11x.</t>
+      </text>
+    </comment>
+    <comment ref="L9" authorId="0" shapeId="0">
+      <text>
+        <t>SM-bound (SM 81% busy; L1/L2 39%, DRAM 0%): SMs x clock 128 x 2.52 / (82 x 1.69) GHz = 2.33x.</t>
+      </text>
+    </comment>
+    <comment ref="L10" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels are 94% of the RTX 3090 time and predicted 2.29x faster; the other 6% (copies, gaps) is unchanged.</t>
+      </text>
+    </comment>
+    <comment ref="L12" authorId="0" shapeId="0">
+      <text>
+        <t>L1/L2-bound (L1/L2 96% busy; SM 7%, DRAM 38%): assumed to scale with SMs x clock, 2.32x.</t>
+      </text>
+    </comment>
+    <comment ref="L13" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels are 70% of the RTX 3090 time and predicted 2.28x faster; the other 30% (copies, gaps) is unchanged.</t>
+      </text>
+    </comment>
+    <comment ref="L15" authorId="0" shapeId="0">
+      <text>
+        <t>DRAM-bound (DRAM 96% busy; SM 10%, L1/L2 96%): data rate 21 / 18.98 Gbps = 1.11x.</t>
+      </text>
+    </comment>
+    <comment ref="L16" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels are 3% of the RTX 3090 time and predicted 1.11x faster; the other 97% (copies, gaps) is unchanged.</t>
+      </text>
+    </comment>
+    <comment ref="L18" authorId="0" shapeId="0">
+      <text>
+        <t>SM-bound (SM 81% busy; L1/L2 76%, DRAM 26%): SMs x clock 128 x 2.52 / (82 x 1.69) GHz = 2.32x.</t>
+      </text>
+    </comment>
+    <comment ref="L19" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels are 10% of the RTX 3090 time and predicted 2.32x faster; the other 90% (copies, gaps) is unchanged.</t>
+      </text>
+    </comment>
+    <comment ref="L21" authorId="0" shapeId="0">
+      <text>
+        <t>DRAM-bound (DRAM 88% busy; SM 3%, L1/L2 88%): data rate 21 / 18.98 Gbps = 1.11x.</t>
+      </text>
+    </comment>
+    <comment ref="L22" authorId="0" shapeId="0">
+      <text>
+        <t>Kernels are 3% of the RTX 3090 time and predicted 1.11x faster; the other 97% (copies, gaps) is unchanged.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1353,7 +1427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1367,8 +1441,9 @@
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1427,11 +1502,11 @@
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Graph speedup
-(Direct / Graph)</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
+          <t>Speedup vs RTX 3090 (CUDA Graph time)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1473,8 +1548,18 @@
           <t>nsys sqlite</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>Predicted</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Measured
+(RTX 3090 / RTX 4090)</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1524,11 +1609,14 @@
           <t>nsys-node-direct-20261015-091935.sqlite</t>
         </is>
       </c>
-      <c r="L6" s="10">
-        <f>IF(AND(ISNUMBER(F6),ISNUMBER(I6)),I6/F6,"")</f>
+      <c r="L6" s="10" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="M6" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F6),ISNUMBER(F6)),'RTX 3090'!F6/F6,"pending")</f>
         <v/>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Largest kernel. It is a matrix-vector product, so its time does not grow with batch; the three kernels run concurrently on separate streams, so their times overlap. </t>
         </is>
@@ -1578,11 +1666,14 @@
           <t>nsys-node-direct-20261015-091935.sqlite</t>
         </is>
       </c>
-      <c r="L7" s="10">
-        <f>IF(AND(ISNUMBER(F7),ISNUMBER(I7)),I7/F7,"")</f>
+      <c r="L7" s="10" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="M7" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F7),ISNUMBER(F7)),'RTX 3090'!F7/F7,"pending")</f>
         <v/>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>Mean of 3 interleaved trials from the GPU-filling sweep; no per-iteration copies. The nsys traces rerun this configuration (963.0 / 962.1 us per iteration).</t>
         </is>
@@ -1632,11 +1723,14 @@
       </c>
       <c r="J9" s="12" t="n"/>
       <c r="K9" s="12" t="n"/>
-      <c r="L9" s="10">
-        <f>IF(AND(ISNUMBER(F9),ISNUMBER(I9)),I9/F9,"")</f>
+      <c r="L9" s="10" t="n">
+        <v>2.325</v>
+      </c>
+      <c r="M9" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F9),ISNUMBER(F9)),'RTX 3090'!F9/F9,"pending")</f>
         <v/>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="N9" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style). </t>
         </is>
@@ -1684,11 +1778,14 @@
       </c>
       <c r="J10" s="12" t="n"/>
       <c r="K10" s="12" t="n"/>
-      <c r="L10" s="10">
-        <f>IF(AND(ISNUMBER(F10),ISNUMBER(I10)),I10/F10,"")</f>
+      <c r="L10" s="10" t="n">
+        <v>2.137</v>
+      </c>
+      <c r="M10" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F10),ISNUMBER(F10)),'RTX 3090'!F10/F10,"pending")</f>
         <v/>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>benchmark.py: median of 5 runs, random inputs. Includes H2D input and D2H output copies.</t>
         </is>
@@ -1738,11 +1835,14 @@
       </c>
       <c r="J12" s="12" t="n"/>
       <c r="K12" s="12" t="n"/>
-      <c r="L12" s="10">
-        <f>IF(AND(ISNUMBER(F12),ISNUMBER(I12)),I12/F12,"")</f>
+      <c r="L12" s="10" t="n">
+        <v>2.323</v>
+      </c>
+      <c r="M12" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F12),ISNUMBER(F12)),'RTX 3090'!F12/F12,"pending")</f>
         <v/>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Pull gather of precomputed contributions. Full-graph iterations only; the first iteration runs as 8 upload-overlapped chunks. </t>
         </is>
@@ -1790,11 +1890,14 @@
       </c>
       <c r="J13" s="12" t="n"/>
       <c r="K13" s="12" t="n"/>
-      <c r="L13" s="10">
-        <f>IF(AND(ISNUMBER(F13),ISNUMBER(I13)),I13/F13,"")</f>
+      <c r="L13" s="10" t="n">
+        <v>1.644</v>
+      </c>
+      <c r="M13" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F13),ISNUMBER(F13)),'RTX 3090'!F13/F13,"pending")</f>
         <v/>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="N13" s="5" t="inlineStr">
         <is>
           <t>Median span of the 1693 replays with transfers in the nsys node trace. The CSR graph is uploaded from pinned memory in 8 chunks overlapped with the first iteration. A separate uninstrumented run of the binary (profiles/bench-20261015-091815.txt): 5.714 ms with transfers, 2.651 ms compute only.</t>
         </is>
@@ -1844,11 +1947,14 @@
       </c>
       <c r="J15" s="12" t="n"/>
       <c r="K15" s="12" t="n"/>
-      <c r="L15" s="10">
-        <f>IF(AND(ISNUMBER(F15),ISNUMBER(I15)),I15/F15,"")</f>
+      <c r="L15" s="10" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="M15" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F15),ISNUMBER(F15)),'RTX 3090'!F15/F15,"pending")</f>
         <v/>
       </c>
-      <c r="M15" s="5" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1892,11 +1998,14 @@
       </c>
       <c r="J16" s="12" t="n"/>
       <c r="K16" s="12" t="n"/>
-      <c r="L16" s="10">
-        <f>IF(AND(ISNUMBER(F16),ISNUMBER(I16)),I16/F16,"")</f>
+      <c r="L16" s="10" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="M16" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F16),ISNUMBER(F16)),'RTX 3090'!F16/F16,"pending")</f>
         <v/>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="N16" s="5" t="inlineStr">
         <is>
           <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
         </is>
@@ -1946,11 +2055,14 @@
       </c>
       <c r="J18" s="12" t="n"/>
       <c r="K18" s="12" t="n"/>
-      <c r="L18" s="10">
-        <f>IF(AND(ISNUMBER(F18),ISNUMBER(I18)),I18/F18,"")</f>
+      <c r="L18" s="10" t="n">
+        <v>2.322</v>
+      </c>
+      <c r="M18" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F18),ISNUMBER(F18)),'RTX 3090'!F18/F18,"pending")</f>
         <v/>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="N18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Only kernel in the application. </t>
         </is>
@@ -1998,11 +2110,14 @@
       </c>
       <c r="J19" s="12" t="n"/>
       <c r="K19" s="12" t="n"/>
-      <c r="L19" s="10">
-        <f>IF(AND(ISNUMBER(F19),ISNUMBER(I19)),I19/F19,"")</f>
+      <c r="L19" s="10" t="n">
+        <v>1.059</v>
+      </c>
+      <c r="M19" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F19),ISNUMBER(F19)),'RTX 3090'!F19/F19,"pending")</f>
         <v/>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
         </is>
@@ -2052,11 +2167,14 @@
       </c>
       <c r="J21" s="12" t="n"/>
       <c r="K21" s="12" t="n"/>
-      <c r="L21" s="10">
-        <f>IF(AND(ISNUMBER(F21),ISNUMBER(I21)),I21/F21,"")</f>
+      <c r="L21" s="10" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="M21" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F21),ISNUMBER(F21)),'RTX 3090'!F21/F21,"pending")</f>
         <v/>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Only kernel in the application. </t>
         </is>
@@ -2104,27 +2222,69 @@
       </c>
       <c r="J22" s="12" t="n"/>
       <c r="K22" s="12" t="n"/>
-      <c r="L22" s="10">
-        <f>IF(AND(ISNUMBER(F22),ISNUMBER(I22)),I22/F22,"")</f>
+      <c r="L22" s="10" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="M22" s="10">
+        <f>IF(AND(ISNUMBER('RTX 3090'!F22),ISNUMBER(F22)),'RTX 3090'!F22/F22,"pending")</f>
         <v/>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="N22" s="5" t="inlineStr">
         <is>
           <t>Median span of the 41 end-to-end replays in the nsys node trace.</t>
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>How the predicted speedup is calculated (hover a Predicted value for that row's reason)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>The predicted speedup uses only the RTX 3090's ncu reports and the two GPUs' published specs (RTX 3090: 82 SMs, 1.695 GHz boost, 19.5 Gbps GDDR6X; RTX 4090: 128 SMs, 2.52 GHz boost, 21 Gbps GDDR6X; both 384-bit, PCIe 4.0 x16), so it is fixed before any 4090 measurement. Each unit's peak scales by its hardware ratio: SM compute by SMs x SM clock, L1/L2 cache throughput assumed to scale the same way, DRAM by memory data rate (the 3090's own SM and memory clocks come from its ncu report: 1.69 GHz and 18.98 Gbps, so the ratios are about 2.32x and 1.11x).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Kernel rows: ncu gives each launch's SM, memory (L1/L2) and DRAM throughput as a percent of the 3090's peak. Keeping the work per unit fixed, a unit at u% that is r times faster needs u/r% of the old time, and the slowest unit sets the new time: speedup = max(u) / max(u / r). So a DRAM-bound kernel gets ~1.11x and a compute- or cache-bound one ~2.32x. A launch below 60% on every unit is latency-bound and gets the SM clock ratio (1.49x). A kernel with several launches combines them weighted by time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Whole-application rows: the kernels in that workload's ncu report (one run of the application) scale by their predicted speedups; the rest of the 3090 time (H2D/D2H copies over the same PCIe 4.0 link, launch gaps) is assumed unchanged. Where the kernels overlap (llama2c's three streams; their summed time exceeds the iteration time), the whole time scales with the kernels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Not modelled: cache capacity (the 4090's L2 is 72 MB vs 6 MB, so data that spilled to DRAM on the 3090 can stay in L2), kernels overlapping copies (pagerank's first iteration), clocks above rated boost, and compiler differences (CUDA 13.3 vs 12.5). Measured = 3090 time / 4090 time for the CUDA Graph column; kernel rows read pending until the 4090 ncu reports exist.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="M4:M5"/>
+  <mergeCells count="14">
+    <mergeCell ref="A27:N27"/>
     <mergeCell ref="B4:B5"/>
+    <mergeCell ref="L4:M4"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A26:N26"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
-    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="A25:N25"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="I4:K4"/>
+    <mergeCell ref="A28:N28"/>
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <hyperlinks>
@@ -2151,6 +2311,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -2181,84 +2342,84 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>ncu report</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Launch #</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Kernel</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>SM throughput %</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Memory throughput %</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>DRAM throughput %</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>Achieved occupancy %</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>Theoretical occupancy %</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>Registers / thread</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>Grid</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="M1" s="15" t="inlineStr">
+      <c r="M1" s="17" t="inlineStr">
         <is>
           <t>Waves / SM</t>
         </is>
       </c>
-      <c r="N1" s="15" t="inlineStr">
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>DRAM read</t>
         </is>
       </c>
-      <c r="O1" s="15" t="inlineStr">
+      <c r="O1" s="17" t="inlineStr">
         <is>
           <t>DRAM write</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2309,7 +2470,7 @@
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2360,7 +2521,7 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2411,7 +2572,7 @@
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2462,7 +2623,7 @@
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2513,7 +2674,7 @@
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2564,7 +2725,7 @@
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2615,7 +2776,7 @@
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2666,7 +2827,7 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-graph-20261014-215130.ncu-rep</t>
         </is>
@@ -2717,7 +2878,7 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2768,7 +2929,7 @@
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2819,7 +2980,7 @@
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2870,7 +3031,7 @@
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2921,7 +3082,7 @@
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -2972,7 +3133,7 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -3023,7 +3184,7 @@
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -3074,7 +3235,7 @@
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -3125,7 +3286,7 @@
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>ncu-large-coalesced-b1024-direct-20261014-215130.ncu-rep</t>
         </is>
@@ -3176,7 +3337,7 @@
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -3227,7 +3388,7 @@
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -3278,7 +3439,7 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -3329,7 +3490,7 @@
       <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>ncu-all-kernels-msa_optimized_large-20260925-142052.ncu-rep</t>
         </is>
@@ -3380,7 +3541,7 @@
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3439,7 +3600,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3498,7 +3659,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3557,7 +3718,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3616,7 +3777,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3675,7 +3836,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3734,7 +3895,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3793,7 +3954,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3852,7 +4013,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3911,7 +4072,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -3970,7 +4131,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4029,7 +4190,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4088,7 +4249,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4147,7 +4308,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="inlineStr">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4206,7 +4367,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4265,7 +4426,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4324,7 +4485,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4383,7 +4544,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="16" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4442,7 +4603,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4501,7 +4662,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4560,7 +4721,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4619,7 +4780,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4678,7 +4839,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4737,7 +4898,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
+      <c r="A47" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4796,7 +4957,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="16" t="inlineStr">
+      <c r="A48" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4855,7 +5016,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4914,7 +5075,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -4973,7 +5134,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>ncu-pagerank-20261007-152417.ncu-rep</t>
         </is>
@@ -5032,7 +5193,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="16" t="inlineStr">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>ncu-anomaly_mse-20261007-144943.ncu-rep</t>
         </is>
@@ -5091,7 +5252,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
+      <c r="A53" s="18" t="inlineStr">
         <is>
           <t>ncu-anomaly_mse-20261007-144943.ncu-rep</t>
         </is>
@@ -5150,7 +5311,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
+      <c r="A54" s="18" t="inlineStr">
         <is>
           <t>ncu-kws_postprocess-20261007-144950.ncu-rep</t>
         </is>
@@ -5209,7 +5370,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
+      <c r="A55" s="18" t="inlineStr">
         <is>
           <t>ncu-vww_preprocess-20261007-144958.ncu-rep</t>
         </is>
@@ -5355,84 +5516,84 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>ncu report</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Launch #</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Kernel</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>Duration</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>SM throughput %</t>
         </is>
       </c>
-      <c r="F1" s="15" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>Memory throughput %</t>
         </is>
       </c>
-      <c r="G1" s="15" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>DRAM throughput %</t>
         </is>
       </c>
-      <c r="H1" s="15" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>Achieved occupancy %</t>
         </is>
       </c>
-      <c r="I1" s="15" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>Theoretical occupancy %</t>
         </is>
       </c>
-      <c r="J1" s="15" t="inlineStr">
+      <c r="J1" s="17" t="inlineStr">
         <is>
           <t>Registers / thread</t>
         </is>
       </c>
-      <c r="K1" s="15" t="inlineStr">
+      <c r="K1" s="17" t="inlineStr">
         <is>
           <t>Grid</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="L1" s="17" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="M1" s="15" t="inlineStr">
+      <c r="M1" s="17" t="inlineStr">
         <is>
           <t>Waves / SM</t>
         </is>
       </c>
-      <c r="N1" s="15" t="inlineStr">
+      <c r="N1" s="17" t="inlineStr">
         <is>
           <t>DRAM read</t>
         </is>
       </c>
-      <c r="O1" s="15" t="inlineStr">
+      <c r="O1" s="17" t="inlineStr">
         <is>
           <t>DRAM write</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>pending (ncu not run yet)</t>
         </is>

</xml_diff>

<commit_message>
Time a launch-bound small shape of every workload on RTX 3090
At the largest shapes an iteration takes milliseconds, so direct launches
and CUDA Graphs match within 1%. time_all.sh now also runs each workload at
a small shape (SHAPES=small, 1000-iteration batches): llama2c with 32
repeats of tiny kernels, loom_msa 4x4, a 2^14-vertex PageRank graph
(make -C pagerank small, PAGERANK_LOG_VERTICES) and the MLPerf smoke sizes.
The spreadsheet gets a small-shape whole-application row per workload
(9 runs on the RTX 3090; pending on the RTX 4090).
</commit_message>
<xml_diff>
--- a/results/cuda_performance.xlsx
+++ b/results/cuda_performance.xlsx
@@ -262,52 +262,52 @@
         <t>Kernels overlap (their summed ncu time is 105% of this time), so all of it scales with the kernels' 1.11x.</t>
       </text>
     </comment>
-    <comment ref="U9" authorId="0" shapeId="0">
+    <comment ref="U10" authorId="0" shapeId="0">
       <text>
         <t>SM-bound (SM 80% busy; L1/L2 39%, DRAM 0%): SMs x clock 128 x 2.52 / (82 x 1.69) GHz = 2.33x.</t>
       </text>
     </comment>
-    <comment ref="U10" authorId="0" shapeId="0">
+    <comment ref="U11" authorId="0" shapeId="0">
       <text>
         <t>Kernels are 95% of the RTX 3090 time and predicted 2.29x faster; the other 5% (copies, gaps) is unchanged.</t>
       </text>
     </comment>
-    <comment ref="U12" authorId="0" shapeId="0">
+    <comment ref="U14" authorId="0" shapeId="0">
       <text>
         <t>L1/L2-bound (L1/L2 96% busy; SM 7%, DRAM 38%): assumed to scale with SMs x clock, 2.32x.</t>
       </text>
     </comment>
-    <comment ref="U13" authorId="0" shapeId="0">
+    <comment ref="U15" authorId="0" shapeId="0">
       <text>
         <t>Kernels are 70% of the RTX 3090 time and predicted 2.29x faster; the other 30% (copies, gaps) is unchanged.</t>
       </text>
     </comment>
-    <comment ref="U15" authorId="0" shapeId="0">
+    <comment ref="U18" authorId="0" shapeId="0">
       <text>
         <t>DRAM-bound (DRAM 96% busy; SM 10%, L1/L2 96%): data rate 21 / 18.98 Gbps = 1.11x.</t>
       </text>
     </comment>
-    <comment ref="U16" authorId="0" shapeId="0">
+    <comment ref="U19" authorId="0" shapeId="0">
       <text>
         <t>Kernels are 3% of the RTX 3090 time and predicted 1.11x faster; the other 97% (copies, gaps) is unchanged.</t>
       </text>
     </comment>
-    <comment ref="U18" authorId="0" shapeId="0">
+    <comment ref="U22" authorId="0" shapeId="0">
       <text>
         <t>SM-bound (SM 81% busy; L1/L2 76%, DRAM 26%): SMs x clock 128 x 2.52 / (82 x 1.69) GHz = 2.33x.</t>
       </text>
     </comment>
-    <comment ref="U19" authorId="0" shapeId="0">
+    <comment ref="U23" authorId="0" shapeId="0">
       <text>
         <t>Kernels are 10% of the RTX 3090 time and predicted 2.33x faster; the other 90% (copies, gaps) is unchanged.</t>
       </text>
     </comment>
-    <comment ref="U21" authorId="0" shapeId="0">
+    <comment ref="U26" authorId="0" shapeId="0">
       <text>
         <t>DRAM-bound (DRAM 88% busy; SM 3%, L1/L2 88%): data rate 21 / 18.98 Gbps = 1.11x.</t>
       </text>
     </comment>
-    <comment ref="U22" authorId="0" shapeId="0">
+    <comment ref="U27" authorId="0" shapeId="0">
       <text>
         <t>Kernels are 3% of the RTX 3090 time and predicted 1.11x faster; the other 97% (copies, gaps) is unchanged.</t>
       </text>
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -648,7 +648,7 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GPU: NVIDIA GeForce RTX 3090 (sm_86, 24 GB), binaries built with CUDA 13.3 (outputs in rtx3090/). Lower is better. Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application, launched directly, as a CUDA Graph, and as the agentic optimized version (&lt;name&gt;_sota.cu, formerly SOTA: the fastest implementation found, same work per iteration, launched whichever way is fastest). Full batch = one batch of back-to-back iterations; per iteration = full batch / iterations; single iteration = median of iterations each launched alone on an idle device, so launch cost is exposed rather than overlapped with the previous iteration. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so kernel rows have one single-launch time.</t>
+          <t>GPU: NVIDIA GeForce RTX 3090 (sm_86, 24 GB), binaries built with CUDA 13.3 (outputs in rtx3090/). Lower is better. Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application, plus the whole application at a small shape where launch cost dominates, launched directly, as a CUDA Graph, and as the agentic optimized version (&lt;name&gt;_sota.cu, formerly SOTA: the fastest implementation found, same work per iteration, launched whichever way is fastest). Full batch = one batch of back-to-back iterations; per iteration = full batch / iterations; single iteration = median of iterations each launched alone on an idle device, so launch cost is exposed rather than overlapped with the previous iteration. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so kernel rows have one single-launch time.</t>
         </is>
       </c>
     </row>
@@ -1061,115 +1061,89 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>loom_msa (multi-sensor attention)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>fuse_attention_kernel</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>25,000 queries x 250,000 context</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>llama2c (coalesced matmul)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>batch=64, dim=256, rows=512, 32 repeats</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>RTX 3090 (sm_86, 24 GB)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="n">
-        <v>8174.176</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>ncu-all-kernels-msa_optimized_large-direct-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>nsys-timing-msa_optimized_large-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="K9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="10" t="n">
-        <v>8174.304</v>
-      </c>
-      <c r="N9" s="11" t="inlineStr">
-        <is>
-          <t>ncu-all-kernels-msa_optimized_large-graph-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
-      <c r="O9" s="11" t="inlineStr">
-        <is>
-          <t>nsys-timing-msa_optimized_large-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="P9" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R9" s="13" t="n">
-        <v>4140.032</v>
-      </c>
-      <c r="S9" s="14" t="inlineStr">
-        <is>
-          <t>ncu-all-kernels-msa_sota_large_1chunk-direct-20261016-145900.ncu-rep</t>
-        </is>
-      </c>
-      <c r="T9" s="14" t="inlineStr">
-        <is>
-          <t>nsys-timing-msa_sota_large-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="U9" s="15" t="n"/>
-      <c r="V9" s="15" t="n">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>112.853</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>112.853</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>113.584</v>
+      </c>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="10" t="n">
+        <v>91.084</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>91.084</v>
+      </c>
+      <c r="M8" s="10" t="n">
+        <v>91.12</v>
+      </c>
+      <c r="N8" s="17" t="n"/>
+      <c r="O8" s="17" t="n"/>
+      <c r="P8" s="13" t="n">
+        <v>70.877</v>
+      </c>
+      <c r="Q8" s="13" t="n">
+        <v>70.877</v>
+      </c>
+      <c r="R8" s="13" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="S8" s="18" t="n"/>
+      <c r="T8" s="18" t="n"/>
+      <c r="U8" s="15" t="n">
+        <v>1.239</v>
+      </c>
+      <c r="V8" s="15" t="n">
+        <v>1.247</v>
+      </c>
+      <c r="W8" s="15" t="n">
+        <v>1.285</v>
+      </c>
+      <c r="X8" s="15" t="n">
+        <v>1.271</v>
+      </c>
+      <c r="Y8" s="15" t="n">
+        <v>1.006</v>
+      </c>
+      <c r="Z8" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="W9" s="15" t="n"/>
-      <c r="X9" s="15" t="n">
-        <v>2.029</v>
-      </c>
-      <c r="Y9" s="15" t="n"/>
-      <c r="Z9" s="15" t="n"/>
-      <c r="AA9" s="15" t="n"/>
-      <c r="AB9" s="5" t="inlineStr">
-        <is>
-          <t>Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style). 93% of the whole-application time per iteration. Agentic optimized (launch=direct): msa_sota_attention_kernel (13-way context split, 8 queries per thread) with the projections folded into its loads and the split merge and statistics into its last block. msa_sota_large runs it as 13 concurrent launches, one per imu copy chunk, which ncu would serialize, so ncu profiles msa_sota_large_1chunk, the same kernel as one launch. Compared with the four graph kernels' summed ncu time (8,400.5 us).</t>
+      <c r="AA8" s="15" t="n">
+        <v>1.011</v>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. One iteration: 32 repeats of rmsnorm + softmax + matmul (96 kernels of about a microsecond each) on device-resident data, no per-iteration copies. Full batch: 1000 back-to-back iterations between CUDA events (per iteration = full batch / 1000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=graph): llama2c_sota_small, the same implementation at this shape.</t>
         </is>
       </c>
     </row>
@@ -1181,91 +1155,203 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>fuse_attention_kernel</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>25,000 queries x 250,000 context</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>8174.176</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>ncu-all-kernels-msa_optimized_large-direct-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>nsys-timing-msa_optimized_large-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="n">
+        <v>8174.304</v>
+      </c>
+      <c r="N10" s="11" t="inlineStr">
+        <is>
+          <t>ncu-all-kernels-msa_optimized_large-graph-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
+      <c r="O10" s="11" t="inlineStr">
+        <is>
+          <t>nsys-timing-msa_optimized_large-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R10" s="13" t="n">
+        <v>4140.032</v>
+      </c>
+      <c r="S10" s="14" t="inlineStr">
+        <is>
+          <t>ncu-all-kernels-msa_sota_large_1chunk-direct-20261016-145900.ncu-rep</t>
+        </is>
+      </c>
+      <c r="T10" s="14" t="inlineStr">
+        <is>
+          <t>nsys-timing-msa_sota_large-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U10" s="15" t="n"/>
+      <c r="V10" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" s="15" t="n"/>
+      <c r="X10" s="15" t="n">
+        <v>2.029</v>
+      </c>
+      <c r="Y10" s="15" t="n"/>
+      <c r="Z10" s="15" t="n"/>
+      <c r="AA10" s="15" t="n"/>
+      <c r="AB10" s="5" t="inlineStr">
+        <is>
+          <t>Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style). 93% of the whole-application time per iteration. Agentic optimized (launch=direct): msa_sota_attention_kernel (13-way context split, 8 queries per thread) with the projections folded into its loads and the split merge and statistics into its last block. msa_sota_large runs it as 13 concurrent launches, one per imu copy chunk, which ncu would serialize, so ncu profiles msa_sota_large_1chunk, the same kernel as one launch. Compared with the four graph kernels' summed ncu time (8,400.5 us).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>loom_msa (multi-sensor attention)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>Whole application (H2D + kernels + D2H)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>25,000 queries x 250,000 context</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>RTX 3090 (sm_86, 24 GB)</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Batch and single iteration (cudaEvent)</t>
         </is>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F11" s="7" t="n">
         <v>441.032</v>
       </c>
-      <c r="G10" s="7" t="n">
+      <c r="G11" s="7" t="n">
         <v>8820.639999999999</v>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H11" s="7" t="n">
         <v>8886.379999999999</v>
       </c>
-      <c r="I10" s="16" t="n"/>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>nsys-timing-msa_optimized_large-direct-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="K10" s="10" t="n">
+      <c r="K11" s="10" t="n">
         <v>440.465</v>
       </c>
-      <c r="L10" s="10" t="n">
+      <c r="L11" s="10" t="n">
         <v>8809.299999999999</v>
       </c>
-      <c r="M10" s="10" t="n">
+      <c r="M11" s="10" t="n">
         <v>8817.58</v>
       </c>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="11" t="inlineStr">
+      <c r="N11" s="17" t="n"/>
+      <c r="O11" s="11" t="inlineStr">
         <is>
           <t>nsys-timing-msa_optimized_large-graph-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="P10" s="13" t="n">
+      <c r="P11" s="13" t="n">
         <v>214.376</v>
       </c>
-      <c r="Q10" s="13" t="n">
+      <c r="Q11" s="13" t="n">
         <v>4287.52</v>
       </c>
-      <c r="R10" s="13" t="n">
+      <c r="R11" s="13" t="n">
         <v>4283.39</v>
       </c>
-      <c r="S10" s="18" t="n"/>
-      <c r="T10" s="14" t="inlineStr">
+      <c r="S11" s="18" t="n"/>
+      <c r="T11" s="14" t="inlineStr">
         <is>
           <t>nsys-timing-msa_sota_large-direct-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="U10" s="15" t="n">
+      <c r="U11" s="15" t="n">
         <v>1.001</v>
       </c>
-      <c r="V10" s="15" t="n">
+      <c r="V11" s="15" t="n">
         <v>1.008</v>
       </c>
-      <c r="W10" s="15" t="n">
+      <c r="W11" s="15" t="n">
         <v>2.055</v>
       </c>
-      <c r="X10" s="15" t="n">
+      <c r="X11" s="15" t="n">
         <v>2.059</v>
       </c>
-      <c r="Y10" s="15" t="n">
+      <c r="Y11" s="15" t="n">
         <v>1.007</v>
       </c>
-      <c r="Z10" s="15" t="n">
+      <c r="Z11" s="15" t="n">
         <v>1.001</v>
       </c>
-      <c r="AA10" s="15" t="n">
+      <c r="AA11" s="15" t="n">
         <v>0.999</v>
       </c>
-      <c r="AB10" s="5" t="inlineStr">
+      <c r="AB11" s="5" t="inlineStr">
         <is>
           <t>msa_optimized_large on random inputs, including the H2D input and D2H output copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): msa_sota_large, rotating over 3 random input sets; output written straight to pinned host memory.</t>
         </is>
@@ -1274,227 +1360,215 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>loom_msa (multi-sensor attention)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>4 queries x 4 context (main.c)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>111.933</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>22.387</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>16.624</v>
+      </c>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="10" t="n">
+        <v>87.453</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>17.491</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <v>14.336</v>
+      </c>
+      <c r="N12" s="17" t="n"/>
+      <c r="O12" s="17" t="n"/>
+      <c r="P12" s="13" t="n">
+        <v>38.76</v>
+      </c>
+      <c r="Q12" s="13" t="n">
+        <v>7.752</v>
+      </c>
+      <c r="R12" s="13" t="n">
+        <v>9.215999999999999</v>
+      </c>
+      <c r="S12" s="18" t="n"/>
+      <c r="T12" s="18" t="n"/>
+      <c r="U12" s="15" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="V12" s="15" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="W12" s="15" t="n">
+        <v>2.256</v>
+      </c>
+      <c r="X12" s="15" t="n">
+        <v>1.556</v>
+      </c>
+      <c r="Y12" s="15" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="Z12" s="15" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AA12" s="15" t="n">
+        <v>1.189</v>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. msa_optimized_4x4 (main.c's shape) on random inputs, including the H2D input and D2H output copies; every copy and kernel moves a few hundred bytes. Full batch: 5000 back-to-back iterations between CUDA events (per iteration = full batch / 5000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=direct): msa_sota_4x4, the same implementation at this shape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>pagerank (GAPBS)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>pagerank_update (one iteration)</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>RTX 3090 (sm_86, 24 GB)</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Kernel time (ncu, one launch)</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H14" s="7" t="n">
         <v>262.621</v>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>ncu-pagerank-direct-20261015-224015.ncu-rep</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>nsys-timing-pagerank-direct-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="K12" s="9" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L12" s="9" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="10" t="n">
+      <c r="M14" s="10" t="n">
         <v>262.754</v>
       </c>
-      <c r="N12" s="11" t="inlineStr">
+      <c r="N14" s="11" t="inlineStr">
         <is>
           <t>ncu-pagerank-graph-20261015-224015.ncu-rep</t>
         </is>
       </c>
-      <c r="O12" s="11" t="inlineStr">
+      <c r="O14" s="11" t="inlineStr">
         <is>
           <t>nsys-timing-pagerank-graph-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="P12" s="12" t="inlineStr">
+      <c r="P14" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R12" s="13" t="n">
+      <c r="R14" s="13" t="n">
         <v>155.326</v>
       </c>
-      <c r="S12" s="14" t="inlineStr">
+      <c r="S14" s="14" t="inlineStr">
         <is>
           <t>ncu-pagerank-sota-direct-20261016-145900.ncu-rep</t>
         </is>
       </c>
-      <c r="T12" s="14" t="inlineStr">
+      <c r="T14" s="14" t="inlineStr">
         <is>
           <t>nsys-timing-pagerank_sota-direct-20261020-161213.sqlite</t>
         </is>
       </c>
-      <c r="U12" s="15" t="n"/>
-      <c r="V12" s="15" t="n">
+      <c r="U14" s="15" t="n"/>
+      <c r="V14" s="15" t="n">
         <v>0.999</v>
       </c>
-      <c r="W12" s="15" t="n"/>
-      <c r="X12" s="15" t="n">
+      <c r="W14" s="15" t="n"/>
+      <c r="X14" s="15" t="n">
         <v>1.692</v>
       </c>
-      <c r="Y12" s="15" t="n"/>
-      <c r="Z12" s="15" t="n"/>
-      <c r="AA12" s="15" t="n"/>
-      <c r="AB12" s="5" t="inlineStr">
+      <c r="Y14" s="15" t="n"/>
+      <c r="Z14" s="15" t="n"/>
+      <c r="AA14" s="15" t="n"/>
+      <c r="AB14" s="5" t="inlineStr">
         <is>
           <t>Pull gather of precomputed contributions. Full-graph iterations only; the first iteration runs as 8 upload-overlapped chunks of ~41 us each. 19 full iterations = 65% of the whole-application time per iteration. Agentic optimized (launch=direct): binned_update_kernel, summed over iterations 1-19 / 19: a cooperative pull over destination parts that fit in shared memory, with edges sorted by source sector on the GPU during the upload (5.4M instead of 16.8M gathered sectors per iteration).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>pagerank (GAPBS)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Whole application (H2D + 20 iterations + D2H)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>RTX 3090 (sm_86, 24 GB)</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Batch and single iteration (cudaEvent)</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>385.722</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>7714.44</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>7662</v>
-      </c>
-      <c r="I13" s="16" t="n"/>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>nsys-timing-pagerank-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="n">
-        <v>382.343</v>
-      </c>
-      <c r="L13" s="10" t="n">
-        <v>7646.86</v>
-      </c>
-      <c r="M13" s="10" t="n">
-        <v>7642</v>
-      </c>
-      <c r="N13" s="17" t="n"/>
-      <c r="O13" s="11" t="inlineStr">
-        <is>
-          <t>nsys-timing-pagerank-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="P13" s="13" t="n">
-        <v>297.939</v>
-      </c>
-      <c r="Q13" s="13" t="n">
-        <v>5958.78</v>
-      </c>
-      <c r="R13" s="13" t="n">
-        <v>5932</v>
-      </c>
-      <c r="S13" s="18" t="n"/>
-      <c r="T13" s="14" t="inlineStr">
-        <is>
-          <t>nsys-timing-pagerank_sota-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="U13" s="15" t="n">
-        <v>1.009</v>
-      </c>
-      <c r="V13" s="15" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="W13" s="15" t="n">
-        <v>1.283</v>
-      </c>
-      <c r="X13" s="15" t="n">
-        <v>1.288</v>
-      </c>
-      <c r="Y13" s="15" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Z13" s="15" t="n">
-        <v>0.999</v>
-      </c>
-      <c r="AA13" s="15" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="AB13" s="5" t="inlineStr">
-        <is>
-          <t>One iteration is one PageRank run: the CSR graph uploaded from pinned memory in 8 chunks overlapped with the first of 20 iterations, then the scores downloaded. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): rotating over 3 inputs (the benchmark graph and two random graphs of the same size); includes the on-GPU edge sort.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny anomaly</t>
+          <t>pagerank (GAPBS)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>mse_partial_kernel</t>
+          <t>Whole application (H2D + 20 iterations + D2H)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>64M elements</t>
+          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1504,109 +1578,95 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>385.722</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>7714.44</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>384.32</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>ncu-anomaly_mse-direct-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
+        <v>7662</v>
+      </c>
+      <c r="I15" s="16" t="n"/>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>nsys-timing-anomaly_mse-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>nsys-timing-pagerank-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K15" s="10" t="n">
+        <v>382.343</v>
+      </c>
+      <c r="L15" s="10" t="n">
+        <v>7646.86</v>
       </c>
       <c r="M15" s="10" t="n">
-        <v>384.288</v>
-      </c>
-      <c r="N15" s="11" t="inlineStr">
-        <is>
-          <t>ncu-anomaly_mse-graph-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
+        <v>7642</v>
+      </c>
+      <c r="N15" s="17" t="n"/>
       <c r="O15" s="11" t="inlineStr">
         <is>
-          <t>nsys-timing-anomaly_mse-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="P15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>nsys-timing-pagerank-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="n">
+        <v>297.939</v>
+      </c>
+      <c r="Q15" s="13" t="n">
+        <v>5958.78</v>
       </c>
       <c r="R15" s="13" t="n">
-        <v>386.24</v>
-      </c>
-      <c r="S15" s="14" t="inlineStr">
-        <is>
-          <t>ncu-anomaly_mse_sota-graph-20261016-145900.ncu-rep</t>
-        </is>
-      </c>
+        <v>5932</v>
+      </c>
+      <c r="S15" s="18" t="n"/>
       <c r="T15" s="14" t="inlineStr">
         <is>
-          <t>nsys-timing-anomaly_mse_sota-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="U15" s="15" t="n"/>
+          <t>nsys-timing-pagerank_sota-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U15" s="15" t="n">
+        <v>1.009</v>
+      </c>
       <c r="V15" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="W15" s="15" t="n"/>
+        <v>1.003</v>
+      </c>
+      <c r="W15" s="15" t="n">
+        <v>1.283</v>
+      </c>
       <c r="X15" s="15" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="Y15" s="15" t="n"/>
-      <c r="Z15" s="15" t="n"/>
-      <c r="AA15" s="15" t="n"/>
+        <v>1.288</v>
+      </c>
+      <c r="Y15" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="Z15" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="AA15" s="15" t="n">
+        <v>0.996</v>
+      </c>
       <c r="AB15" s="5" t="inlineStr">
         <is>
-          <t>3% of the whole-application time per iteration. Agentic optimized (launch=graph): mse_sota_kernel, one single-pass reduction (the last block finishes the sum), compared with mse_partial_kernel + mse_finalize_kernel.</t>
+          <t>One iteration is one PageRank run: the CSR graph uploaded from pinned memory in 8 chunks overlapped with the first of 20 iterations, then the scores downloaded. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): rotating over 3 inputs (the benchmark graph and two random graphs of the same size); includes the on-GPU edge sort.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny anomaly</t>
+          <t>pagerank (GAPBS)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Whole application (H2D + kernels + D2H)</t>
+          <t>Whole application, small shape (launch-bound)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>64M elements</t>
+          <t>2^14 vertices, 16 edges/vertex, 20 iterations</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1620,91 +1680,79 @@
         </is>
       </c>
       <c r="F16" s="7" t="n">
-        <v>708.449</v>
+        <v>168.731</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>14168.98</v>
+        <v>168.731</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>14165.36</v>
+        <v>170</v>
       </c>
       <c r="I16" s="16" t="n"/>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>nsys-timing-anomaly_mse-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
+      <c r="J16" s="16" t="n"/>
       <c r="K16" s="10" t="n">
-        <v>708.564</v>
+        <v>159.4</v>
       </c>
       <c r="L16" s="10" t="n">
-        <v>14171.28</v>
+        <v>159.4</v>
       </c>
       <c r="M16" s="10" t="n">
-        <v>14163.28</v>
+        <v>156</v>
       </c>
       <c r="N16" s="17" t="n"/>
-      <c r="O16" s="11" t="inlineStr">
-        <is>
-          <t>nsys-timing-anomaly_mse-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
+      <c r="O16" s="17" t="n"/>
       <c r="P16" s="13" t="n">
-        <v>691.636</v>
+        <v>602.149</v>
       </c>
       <c r="Q16" s="13" t="n">
-        <v>13832.72</v>
+        <v>602.149</v>
       </c>
       <c r="R16" s="13" t="n">
-        <v>13830.608</v>
+        <v>605</v>
       </c>
       <c r="S16" s="18" t="n"/>
-      <c r="T16" s="14" t="inlineStr">
-        <is>
-          <t>nsys-timing-anomaly_mse_sota-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
+      <c r="T16" s="18" t="n"/>
       <c r="U16" s="15" t="n">
-        <v>1</v>
+        <v>1.059</v>
       </c>
       <c r="V16" s="15" t="n">
-        <v>1</v>
+        <v>1.09</v>
       </c>
       <c r="W16" s="15" t="n">
-        <v>1.024</v>
+        <v>0.265</v>
       </c>
       <c r="X16" s="15" t="n">
-        <v>1.024</v>
+        <v>0.258</v>
       </c>
       <c r="Y16" s="15" t="n">
-        <v>1</v>
+        <v>1.008</v>
       </c>
       <c r="Z16" s="15" t="n">
-        <v>0.999</v>
+        <v>0.979</v>
       </c>
       <c r="AA16" s="15" t="n">
-        <v>1</v>
+        <v>1.005</v>
       </c>
       <c r="AB16" s="5" t="inlineStr">
         <is>
-          <t>Random inputs, including the H2D and D2H copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=graph): rotating over 3 inputs; the float input is copied in shrinking chunks while a second stream reduces each chunk as it lands; the result is written straight to pinned host memory.</t>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The same PageRank run on a 2^14-vertex graph (make -C pagerank small): upload, 20 iterations of a few microseconds each, download. Full batch: 1000 back-to-back iterations between CUDA events (per iteration = full batch / 1000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=direct): pagerank_sota_small, the same implementation at this shape.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny KWS</t>
+          <t>mlperf-tiny anomaly</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>kws_postprocess_kernel</t>
+          <t>mse_partial_kernel</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>12 classes x 4M rows</t>
+          <t>64M elements</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -1728,16 +1776,16 @@
         </is>
       </c>
       <c r="H18" s="7" t="n">
-        <v>1119.968</v>
+        <v>384.32</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>ncu-kws_postprocess-direct-20261015-224015.ncu-rep</t>
+          <t>ncu-anomaly_mse-direct-20261015-224015.ncu-rep</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess-direct-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse-direct-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
@@ -1751,16 +1799,16 @@
         </is>
       </c>
       <c r="M18" s="10" t="n">
-        <v>1120.224</v>
+        <v>384.288</v>
       </c>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>ncu-kws_postprocess-graph-20261015-224015.ncu-rep</t>
+          <t>ncu-anomaly_mse-graph-20261015-224015.ncu-rep</t>
         </is>
       </c>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess-graph-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse-graph-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="P18" s="12" t="inlineStr">
@@ -1774,16 +1822,16 @@
         </is>
       </c>
       <c r="R18" s="13" t="n">
-        <v>323.072</v>
+        <v>386.24</v>
       </c>
       <c r="S18" s="14" t="inlineStr">
         <is>
-          <t>ncu-kws_postprocess_sota-direct-20261016-145900.ncu-rep</t>
+          <t>ncu-anomaly_mse_sota-graph-20261016-145900.ncu-rep</t>
         </is>
       </c>
       <c r="T18" s="14" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess_sota-direct-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse_sota-graph-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="U18" s="15" t="n"/>
@@ -1792,21 +1840,21 @@
       </c>
       <c r="W18" s="15" t="n"/>
       <c r="X18" s="15" t="n">
-        <v>3.467</v>
+        <v>1.003</v>
       </c>
       <c r="Y18" s="15" t="n"/>
       <c r="Z18" s="15" t="n"/>
       <c r="AA18" s="15" t="n"/>
       <c r="AB18" s="5" t="inlineStr">
         <is>
-          <t>Only kernel in the application. 10% of the whole-application time per iteration. Agentic optimized (launch=direct): kws_postprocess_sota_kernel on device buffers (kernels-only), one row per thread with rows staged through shared memory for coalesced 16 B loads and stores.</t>
+          <t>3% of the whole-application time per iteration. Agentic optimized (launch=graph): mse_sota_kernel, one single-pass reduction (the last block finishes the sum), compared with mse_partial_kernel + mse_finalize_kernel.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny KWS</t>
+          <t>mlperf-tiny anomaly</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1816,7 +1864,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>12 classes x 4M rows</t>
+          <t>64M elements</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1830,48 +1878,48 @@
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>568.751</v>
+        <v>708.449</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>11375.02</v>
+        <v>14168.98</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>11370.864</v>
+        <v>14165.36</v>
       </c>
       <c r="I19" s="16" t="n"/>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess-direct-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse-direct-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="K19" s="10" t="n">
-        <v>568.535</v>
+        <v>708.564</v>
       </c>
       <c r="L19" s="10" t="n">
-        <v>11370.7</v>
+        <v>14171.28</v>
       </c>
       <c r="M19" s="10" t="n">
-        <v>11376.016</v>
+        <v>14163.28</v>
       </c>
       <c r="N19" s="17" t="n"/>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess-graph-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse-graph-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="P19" s="13" t="n">
-        <v>433.252</v>
+        <v>691.636</v>
       </c>
       <c r="Q19" s="13" t="n">
-        <v>8665.040000000001</v>
+        <v>13832.72</v>
       </c>
       <c r="R19" s="13" t="n">
-        <v>8654.575999999999</v>
+        <v>13830.608</v>
       </c>
       <c r="S19" s="18" t="n"/>
       <c r="T19" s="14" t="inlineStr">
         <is>
-          <t>nsys-timing-kws_postprocess_sota-direct-20261020-161213.sqlite</t>
+          <t>nsys-timing-anomaly_mse_sota-graph-20261020-161213.sqlite</t>
         </is>
       </c>
       <c r="U19" s="15" t="n">
@@ -1881,152 +1929,126 @@
         <v>1</v>
       </c>
       <c r="W19" s="15" t="n">
-        <v>1.312</v>
+        <v>1.024</v>
       </c>
       <c r="X19" s="15" t="n">
-        <v>1.314</v>
+        <v>1.024</v>
       </c>
       <c r="Y19" s="15" t="n">
         <v>1</v>
       </c>
       <c r="Z19" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="AA19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AA19" s="15" t="n">
-        <v>0.999</v>
-      </c>
       <c r="AB19" s="5" t="inlineStr">
         <is>
-          <t>Random inputs, including the H2D and D2H copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): rotating over 3 inputs; one zero-copy kernel reads the int8 rows from and writes the probabilities and argmax to mapped pinned host memory, so both PCIe directions stream at once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>mlperf-tiny VWW</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>vww_preprocess_kernel</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>256M bytes</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+          <t>Random inputs, including the H2D and D2H copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=graph): rotating over 3 inputs; the float input is copied in shrinking chunks while a second stream reduces each chunk as it lands; the result is written straight to pinned host memory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny anomaly</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>16 elements (smoke)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>RTX 3090 (sm_86, 24 GB)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>659.456</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>ncu-vww_preprocess-direct-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>nsys-timing-vww_preprocess-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="K21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M21" s="10" t="n">
-        <v>664.96</v>
-      </c>
-      <c r="N21" s="11" t="inlineStr">
-        <is>
-          <t>ncu-vww_preprocess-graph-20261015-224015.ncu-rep</t>
-        </is>
-      </c>
-      <c r="O21" s="11" t="inlineStr">
-        <is>
-          <t>nsys-timing-vww_preprocess-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="P21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R21" s="13" t="n">
-        <v>634.72</v>
-      </c>
-      <c r="S21" s="14" t="inlineStr">
-        <is>
-          <t>ncu-vww_preprocess_sota-direct-20261016-145900.ncu-rep</t>
-        </is>
-      </c>
-      <c r="T21" s="14" t="inlineStr">
-        <is>
-          <t>nsys-timing-vww_preprocess_sota-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="U21" s="15" t="n"/>
-      <c r="V21" s="15" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="W21" s="15" t="n"/>
-      <c r="X21" s="15" t="n">
-        <v>1.048</v>
-      </c>
-      <c r="Y21" s="15" t="n"/>
-      <c r="Z21" s="15" t="n"/>
-      <c r="AA21" s="15" t="n"/>
-      <c r="AB21" s="5" t="inlineStr">
-        <is>
-          <t>Only kernel in the application. 3% of the whole-application time per iteration. Agentic optimized (launch=direct): vww_preprocess_sota_kernel on device buffers (kernels-only), four 16 B vectors per thread.</t>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>17.533</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>17.533</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>13.616</v>
+      </c>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="10" t="n">
+        <v>17.393</v>
+      </c>
+      <c r="L20" s="10" t="n">
+        <v>17.393</v>
+      </c>
+      <c r="M20" s="10" t="n">
+        <v>20.272</v>
+      </c>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="17" t="n"/>
+      <c r="P20" s="13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="Q20" s="13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="R20" s="13" t="n">
+        <v>4.096</v>
+      </c>
+      <c r="S20" s="18" t="n"/>
+      <c r="T20" s="18" t="n"/>
+      <c r="U20" s="15" t="n">
+        <v>1.008</v>
+      </c>
+      <c r="V20" s="15" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="W20" s="15" t="n">
+        <v>5.352</v>
+      </c>
+      <c r="X20" s="15" t="n">
+        <v>4.949</v>
+      </c>
+      <c r="Y20" s="15" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="Z20" s="15" t="n">
+        <v>1.166</v>
+      </c>
+      <c r="AA20" s="15" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AB20" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each. Full batch: 1000 back-to-back iterations between CUDA events (per iteration = full batch / 1000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=graph): anomaly_mse_sota_small, the same implementation at this shape.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny VWW</t>
+          <t>mlperf-tiny KWS</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Whole application (H2D + kernels + D2H)</t>
+          <t>kws_postprocess_kernel</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>256M bytes</t>
+          <t>12 classes x 4M rows</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2036,78 +2058,572 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Batch and single iteration (cudaEvent)</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>1094.1</v>
-      </c>
-      <c r="G22" s="7" t="n">
-        <v>21882</v>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="H22" s="7" t="n">
-        <v>21881.408</v>
-      </c>
-      <c r="I22" s="16" t="n"/>
+        <v>1119.968</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>ncu-kws_postprocess-direct-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>nsys-timing-vww_preprocess-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="n">
-        <v>1093.995</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>21879.9</v>
+          <t>nsys-timing-kws_postprocess-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M22" s="10" t="n">
-        <v>21880.512</v>
-      </c>
-      <c r="N22" s="17" t="n"/>
+        <v>1120.224</v>
+      </c>
+      <c r="N22" s="11" t="inlineStr">
+        <is>
+          <t>ncu-kws_postprocess-graph-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>nsys-timing-vww_preprocess-graph-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="P22" s="13" t="n">
-        <v>613.24</v>
-      </c>
-      <c r="Q22" s="13" t="n">
-        <v>12264.8</v>
+          <t>nsys-timing-kws_postprocess-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P22" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="R22" s="13" t="n">
-        <v>12253.552</v>
-      </c>
-      <c r="S22" s="18" t="n"/>
+        <v>323.072</v>
+      </c>
+      <c r="S22" s="14" t="inlineStr">
+        <is>
+          <t>ncu-kws_postprocess_sota-direct-20261016-145900.ncu-rep</t>
+        </is>
+      </c>
       <c r="T22" s="14" t="inlineStr">
         <is>
-          <t>nsys-timing-vww_preprocess_sota-direct-20261020-161213.sqlite</t>
-        </is>
-      </c>
-      <c r="U22" s="15" t="n">
-        <v>1</v>
-      </c>
+          <t>nsys-timing-kws_postprocess_sota-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U22" s="15" t="n"/>
       <c r="V22" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="W22" s="15" t="n">
+      <c r="W22" s="15" t="n"/>
+      <c r="X22" s="15" t="n">
+        <v>3.467</v>
+      </c>
+      <c r="Y22" s="15" t="n"/>
+      <c r="Z22" s="15" t="n"/>
+      <c r="AA22" s="15" t="n"/>
+      <c r="AB22" s="5" t="inlineStr">
+        <is>
+          <t>Only kernel in the application. 10% of the whole-application time per iteration. Agentic optimized (launch=direct): kws_postprocess_sota_kernel on device buffers (kernels-only), one row per thread with rows staged through shared memory for coalesced 16 B loads and stores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 4M rows</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>568.751</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>11375.02</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>11370.864</v>
+      </c>
+      <c r="I23" s="16" t="n"/>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>nsys-timing-kws_postprocess-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>568.535</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>11370.7</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>11376.016</v>
+      </c>
+      <c r="N23" s="17" t="n"/>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>nsys-timing-kws_postprocess-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P23" s="13" t="n">
+        <v>433.252</v>
+      </c>
+      <c r="Q23" s="13" t="n">
+        <v>8665.040000000001</v>
+      </c>
+      <c r="R23" s="13" t="n">
+        <v>8654.575999999999</v>
+      </c>
+      <c r="S23" s="18" t="n"/>
+      <c r="T23" s="14" t="inlineStr">
+        <is>
+          <t>nsys-timing-kws_postprocess_sota-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W23" s="15" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="X23" s="15" t="n">
+        <v>1.314</v>
+      </c>
+      <c r="Y23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA23" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="AB23" s="5" t="inlineStr">
+        <is>
+          <t>Random inputs, including the H2D and D2H copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): rotating over 3 inputs; one zero-copy kernel reads the int8 rows from and writes the probabilities and argmax to mapped pinned host memory, so both PCIe directions stream at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 1 row (smoke)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>10.668</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>10.668</v>
+      </c>
+      <c r="H24" s="7" t="n">
+        <v>20.832</v>
+      </c>
+      <c r="I24" s="16" t="n"/>
+      <c r="J24" s="16" t="n"/>
+      <c r="K24" s="10" t="n">
+        <v>9.369</v>
+      </c>
+      <c r="L24" s="10" t="n">
+        <v>9.369</v>
+      </c>
+      <c r="M24" s="10" t="n">
+        <v>20.752</v>
+      </c>
+      <c r="N24" s="17" t="n"/>
+      <c r="O24" s="17" t="n"/>
+      <c r="P24" s="13" t="n">
+        <v>2.838</v>
+      </c>
+      <c r="Q24" s="13" t="n">
+        <v>2.838</v>
+      </c>
+      <c r="R24" s="13" t="n">
+        <v>4.096</v>
+      </c>
+      <c r="S24" s="18" t="n"/>
+      <c r="T24" s="18" t="n"/>
+      <c r="U24" s="15" t="n">
+        <v>1.139</v>
+      </c>
+      <c r="V24" s="15" t="n">
+        <v>1.004</v>
+      </c>
+      <c r="W24" s="15" t="n">
+        <v>3.301</v>
+      </c>
+      <c r="X24" s="15" t="n">
+        <v>5.066</v>
+      </c>
+      <c r="Y24" s="15" t="n">
+        <v>1.953</v>
+      </c>
+      <c r="Z24" s="15" t="n">
+        <v>2.215</v>
+      </c>
+      <c r="AA24" s="15" t="n">
+        <v>1.443</v>
+      </c>
+      <c r="AB24" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each. Full batch: 1000 back-to-back iterations between CUDA events (per iteration = full batch / 1000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=direct): kws_postprocess_sota_small, the same implementation at this shape.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>vww_preprocess_kernel</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="n">
+        <v>659.456</v>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>ncu-vww_preprocess-direct-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="10" t="n">
+        <v>664.96</v>
+      </c>
+      <c r="N26" s="11" t="inlineStr">
+        <is>
+          <t>ncu-vww_preprocess-graph-20261015-224015.ncu-rep</t>
+        </is>
+      </c>
+      <c r="O26" s="11" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q26" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R26" s="13" t="n">
+        <v>634.72</v>
+      </c>
+      <c r="S26" s="14" t="inlineStr">
+        <is>
+          <t>ncu-vww_preprocess_sota-direct-20261016-145900.ncu-rep</t>
+        </is>
+      </c>
+      <c r="T26" s="14" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess_sota-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U26" s="15" t="n"/>
+      <c r="V26" s="15" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="W26" s="15" t="n"/>
+      <c r="X26" s="15" t="n">
+        <v>1.048</v>
+      </c>
+      <c r="Y26" s="15" t="n"/>
+      <c r="Z26" s="15" t="n"/>
+      <c r="AA26" s="15" t="n"/>
+      <c r="AB26" s="5" t="inlineStr">
+        <is>
+          <t>Only kernel in the application. 3% of the whole-application time per iteration. Agentic optimized (launch=direct): vww_preprocess_sota_kernel on device buffers (kernels-only), four 16 B vectors per thread.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>1094.1</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>21882</v>
+      </c>
+      <c r="H27" s="7" t="n">
+        <v>21881.408</v>
+      </c>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="K27" s="10" t="n">
+        <v>1093.995</v>
+      </c>
+      <c r="L27" s="10" t="n">
+        <v>21879.9</v>
+      </c>
+      <c r="M27" s="10" t="n">
+        <v>21880.512</v>
+      </c>
+      <c r="N27" s="17" t="n"/>
+      <c r="O27" s="11" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess-graph-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="P27" s="13" t="n">
+        <v>613.24</v>
+      </c>
+      <c r="Q27" s="13" t="n">
+        <v>12264.8</v>
+      </c>
+      <c r="R27" s="13" t="n">
+        <v>12253.552</v>
+      </c>
+      <c r="S27" s="18" t="n"/>
+      <c r="T27" s="14" t="inlineStr">
+        <is>
+          <t>nsys-timing-vww_preprocess_sota-direct-20261020-161213.sqlite</t>
+        </is>
+      </c>
+      <c r="U27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" s="15" t="n">
         <v>1.784</v>
       </c>
-      <c r="X22" s="15" t="n">
+      <c r="X27" s="15" t="n">
         <v>1.786</v>
       </c>
-      <c r="Y22" s="15" t="n">
+      <c r="Y27" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="Z22" s="15" t="n">
+      <c r="Z27" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AA22" s="15" t="n">
+      <c r="AA27" s="15" t="n">
         <v>0.999</v>
       </c>
-      <c r="AB22" s="5" t="inlineStr">
+      <c r="AB27" s="5" t="inlineStr">
         <is>
           <t>Random inputs, including the H2D and D2H copies. Full batch: 50 back-to-back iterations between CUDA events (per iteration = full batch / 50). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 5 interleaved runs (time_all.sh). Agentic optimized (launch=direct): rotating over 3 inputs; 64 chunks of 4 MiB on separate copy-in, compute and copy-out streams, so H2D and D2H overlap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>16 bytes (smoke)</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>RTX 3090 (sm_86, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>8.733000000000001</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>8.733000000000001</v>
+      </c>
+      <c r="H28" s="7" t="n">
+        <v>19.76</v>
+      </c>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="16" t="n"/>
+      <c r="K28" s="10" t="n">
+        <v>8.074999999999999</v>
+      </c>
+      <c r="L28" s="10" t="n">
+        <v>8.074999999999999</v>
+      </c>
+      <c r="M28" s="10" t="n">
+        <v>19.776</v>
+      </c>
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="17" t="n"/>
+      <c r="P28" s="13" t="n">
+        <v>12.097</v>
+      </c>
+      <c r="Q28" s="13" t="n">
+        <v>12.097</v>
+      </c>
+      <c r="R28" s="13" t="n">
+        <v>21.376</v>
+      </c>
+      <c r="S28" s="18" t="n"/>
+      <c r="T28" s="18" t="n"/>
+      <c r="U28" s="15" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="V28" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="W28" s="15" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="X28" s="15" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="Y28" s="15" t="n">
+        <v>2.263</v>
+      </c>
+      <c r="Z28" s="15" t="n">
+        <v>2.449</v>
+      </c>
+      <c r="AA28" s="15" t="n">
+        <v>1.767</v>
+      </c>
+      <c r="AB28" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each. Full batch: 1000 back-to-back iterations between CUDA events (per iteration = full batch / 1000). Single iteration: median of 20 iterations, each launched alone on an idle device, so its launch cost is not hidden behind the previous iteration's work. Each time is the median of 9 interleaved runs (time_all.sh). Agentic optimized (launch=direct): vww_preprocess_sota_small, the same implementation at this shape.</t>
         </is>
       </c>
     </row>
@@ -2149,111 +2665,165 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R7" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T7" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R9" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T9" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T12" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R13" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T13" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T16" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T19" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R21" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T21" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R8" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R10" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T10" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R11" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T11" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R12" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R14" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T14" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P15" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R15" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T15" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P16" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R16" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R18" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T18" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P19" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R19" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T19" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P20" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R20" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R22" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T22" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R23" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T23" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R24" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N26" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R26" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T26" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P27" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R27" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="T27" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P28" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="R28" r:id="rId180"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2265,7 +2835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y28"/>
+  <dimension ref="A1:Y34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2305,7 +2875,7 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GPU: NVIDIA GeForce RTX 4090 (sm_89, 24 GB), binaries built with CUDA 12.5 (outputs in rtx4090/). Lower is better. Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application, launched directly, as a CUDA Graph, and as the agentic optimized version (&lt;name&gt;_sota.cu, formerly SOTA: the fastest implementation found, same work per iteration, launched whichever way is fastest). Full batch = one batch of back-to-back iterations; per iteration = full batch / iterations; single iteration = median of iterations each launched alone on an idle device, so launch cost is exposed rather than overlapped with the previous iteration. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so kernel rows have one single-launch time.</t>
+          <t>GPU: NVIDIA GeForce RTX 4090 (sm_89, 24 GB), binaries built with CUDA 12.5 (outputs in rtx4090/). Lower is better. Latest run of each workload's current implementation at the largest problem size tested: the dominant kernel (if one dominates) and the whole application, plus the whole application at a small shape where launch cost dominates, launched directly, as a CUDA Graph, and as the agentic optimized version (&lt;name&gt;_sota.cu, formerly SOTA: the fastest implementation found, same work per iteration, launched whichever way is fastest). Full batch = one batch of back-to-back iterations; per iteration = full batch / iterations; single iteration = median of iterations each launched alone on an idle device, so launch cost is exposed rather than overlapped with the previous iteration. Each value links to its source; the ncu-rep / nsys sqlite columns link the profile files on GitHub. ncu replays each kernel in isolation, so kernel rows have one single-launch time.</t>
         </is>
       </c>
     </row>
@@ -2674,99 +3244,69 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>loom_msa (multi-sensor attention)</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>fuse_attention_kernel</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>25,000 queries x 250,000 context</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>llama2c (coalesced matmul)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>batch=64, dim=256, rows=512, 32 repeats</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>RTX 4090 (sm_89, 24 GB)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>pending (direct mode not profiled yet)</t>
-        </is>
-      </c>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="9" t="inlineStr">
-        <is>
-          <t>pending (ncu not run yet)</t>
-        </is>
-      </c>
-      <c r="N9" s="17" t="n"/>
-      <c r="O9" s="11" t="inlineStr">
-        <is>
-          <t>nsys-msa_optimized_large-20261015-091307.sqlite</t>
-        </is>
-      </c>
-      <c r="P9" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R9" s="12" t="inlineStr">
-        <is>
-          <t>pending (agentic optimized not profiled yet)</t>
-        </is>
-      </c>
-      <c r="S9" s="18" t="n"/>
-      <c r="T9" s="18" t="n"/>
-      <c r="U9" s="15" t="n">
-        <v>2.327</v>
-      </c>
-      <c r="V9" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!M9),ISNUMBER(M9)),'RTX 3090'!M9/M9,"pending")</f>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="16" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="M8" s="17" t="n"/>
+      <c r="N8" s="17" t="n"/>
+      <c r="O8" s="17" t="n"/>
+      <c r="P8" s="18" t="n"/>
+      <c r="Q8" s="12" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="R8" s="18" t="n"/>
+      <c r="S8" s="18" t="n"/>
+      <c r="T8" s="18" t="n"/>
+      <c r="U8" s="15" t="n"/>
+      <c r="V8" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L8),ISNUMBER(L8)),'RTX 3090'!L8/L8,"pending")</f>
         <v/>
       </c>
-      <c r="W9" s="15" t="n"/>
-      <c r="X9" s="15" t="n"/>
-      <c r="Y9" s="5" t="inlineStr">
-        <is>
-          <t>Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style).</t>
+      <c r="W8" s="15" t="n"/>
+      <c r="X8" s="15" t="n"/>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. One iteration: 32 repeats of rmsnorm + softmax + matmul (96 kernels of about a microsecond each) on device-resident data, no per-iteration copies.</t>
         </is>
       </c>
     </row>
@@ -2778,7 +3318,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Whole application (H2D + kernels + D2H)</t>
+          <t>fuse_attention_kernel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -2793,29 +3333,39 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Iteration time (cudaEvent)</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="n"/>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
           <t>pending (direct mode not profiled yet)</t>
         </is>
       </c>
-      <c r="H10" s="16" t="n"/>
       <c r="I10" s="16" t="n"/>
       <c r="J10" s="16" t="n"/>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>pending (time_all.sh not run yet)</t>
-        </is>
-      </c>
-      <c r="L10" s="10" t="n">
-        <v>3835.57</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>pending (time_all.sh not run yet)</t>
+          <t>pending (ncu not run yet)</t>
         </is>
       </c>
       <c r="N10" s="17" t="n"/>
@@ -2824,26 +3374,112 @@
           <t>nsys-msa_optimized_large-20261015-091307.sqlite</t>
         </is>
       </c>
-      <c r="P10" s="18" t="n"/>
+      <c r="P10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q10" s="12" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
+        <is>
           <t>pending (agentic optimized not profiled yet)</t>
         </is>
       </c>
-      <c r="R10" s="18" t="n"/>
       <c r="S10" s="18" t="n"/>
       <c r="T10" s="18" t="n"/>
       <c r="U10" s="15" t="n">
-        <v>2.162</v>
+        <v>2.327</v>
       </c>
       <c r="V10" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!L10),ISNUMBER(L10)),'RTX 3090'!L10/L10,"pending")</f>
+        <f>IF(AND(ISNUMBER('RTX 3090'!M10),ISNUMBER(M10)),'RTX 3090'!M10/M10,"pending")</f>
         <v/>
       </c>
       <c r="W10" s="15" t="n"/>
       <c r="X10" s="15" t="n"/>
       <c r="Y10" s="5" t="inlineStr">
         <is>
+          <t>Single-pass online softmax, shared-memory context tiles, 8-way context split (FlashAttention-style).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>loom_msa (multi-sensor attention)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>25,000 queries x 250,000 context</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Iteration time (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>pending (direct mode not profiled yet)</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="16" t="n"/>
+      <c r="K11" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>3835.57</v>
+      </c>
+      <c r="M11" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="n"/>
+      <c r="O11" s="11" t="inlineStr">
+        <is>
+          <t>nsys-msa_optimized_large-20261015-091307.sqlite</t>
+        </is>
+      </c>
+      <c r="P11" s="18" t="n"/>
+      <c r="Q11" s="12" t="inlineStr">
+        <is>
+          <t>pending (agentic optimized not profiled yet)</t>
+        </is>
+      </c>
+      <c r="R11" s="18" t="n"/>
+      <c r="S11" s="18" t="n"/>
+      <c r="T11" s="18" t="n"/>
+      <c r="U11" s="15" t="n">
+        <v>2.162</v>
+      </c>
+      <c r="V11" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L11),ISNUMBER(L11)),'RTX 3090'!L11/L11,"pending")</f>
+        <v/>
+      </c>
+      <c r="W11" s="15" t="n"/>
+      <c r="X11" s="15" t="n"/>
+      <c r="Y11" s="5" t="inlineStr">
+        <is>
           <t>benchmark.py: median of 5 runs, random inputs, CUDA graph only. Includes H2D input and D2H output copies.</t>
         </is>
       </c>
@@ -2851,17 +3487,17 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>pagerank (GAPBS)</t>
+          <t>loom_msa (multi-sensor attention)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>pagerank_update (one iteration)</t>
+          <t>Whole application, small shape (launch-bound)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
+          <t>4 queries x 4 context (main.c)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -2871,171 +3507,159 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="n"/>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>pending (direct mode not profiled yet)</t>
-        </is>
-      </c>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="n"/>
       <c r="I12" s="16" t="n"/>
       <c r="J12" s="16" t="n"/>
-      <c r="K12" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="K12" s="17" t="n"/>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M12" s="9" t="inlineStr">
-        <is>
-          <t>pending (ncu not run yet)</t>
-        </is>
-      </c>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="n"/>
       <c r="N12" s="17" t="n"/>
-      <c r="O12" s="11" t="inlineStr">
-        <is>
-          <t>nsys-20261015-091708.sqlite</t>
-        </is>
-      </c>
-      <c r="P12" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O12" s="17" t="n"/>
+      <c r="P12" s="18" t="n"/>
       <c r="Q12" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R12" s="12" t="inlineStr">
-        <is>
-          <t>pending (agentic optimized not profiled yet)</t>
-        </is>
-      </c>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="R12" s="18" t="n"/>
       <c r="S12" s="18" t="n"/>
       <c r="T12" s="18" t="n"/>
-      <c r="U12" s="15" t="n">
-        <v>2.325</v>
-      </c>
+      <c r="U12" s="15" t="n"/>
       <c r="V12" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!M12),ISNUMBER(M12)),'RTX 3090'!M12/M12,"pending")</f>
+        <f>IF(AND(ISNUMBER('RTX 3090'!L12),ISNUMBER(L12)),'RTX 3090'!L12/L12,"pending")</f>
         <v/>
       </c>
       <c r="W12" s="15" t="n"/>
       <c r="X12" s="15" t="n"/>
       <c r="Y12" s="5" t="inlineStr">
         <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. msa_optimized_4x4 (main.c's shape) on random inputs, including the H2D input and D2H output copies; every copy and kernel moves a few hundred bytes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>pagerank (GAPBS)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>pagerank_update (one iteration)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>pending (direct mode not profiled yet)</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="n"/>
+      <c r="J14" s="16" t="n"/>
+      <c r="K14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="9" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="n"/>
+      <c r="O14" s="11" t="inlineStr">
+        <is>
+          <t>nsys-20261015-091708.sqlite</t>
+        </is>
+      </c>
+      <c r="P14" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R14" s="12" t="inlineStr">
+        <is>
+          <t>pending (agentic optimized not profiled yet)</t>
+        </is>
+      </c>
+      <c r="S14" s="18" t="n"/>
+      <c r="T14" s="18" t="n"/>
+      <c r="U14" s="15" t="n">
+        <v>2.325</v>
+      </c>
+      <c r="V14" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!M14),ISNUMBER(M14)),'RTX 3090'!M14/M14,"pending")</f>
+        <v/>
+      </c>
+      <c r="W14" s="15" t="n"/>
+      <c r="X14" s="15" t="n"/>
+      <c r="Y14" s="5" t="inlineStr">
+        <is>
           <t>Pull gather of precomputed contributions. Full-graph iterations only; the first iteration runs as 8 upload-overlapped chunks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>pagerank (GAPBS)</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Whole application (H2D + 20 iterations + D2H)</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>RTX 4090 (sm_89, 24 GB)</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Iteration time (nsys)</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>pending (direct mode not profiled yet)</t>
-        </is>
-      </c>
-      <c r="H13" s="16" t="n"/>
-      <c r="I13" s="16" t="n"/>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="9" t="inlineStr">
-        <is>
-          <t>pending (time_all.sh not run yet)</t>
-        </is>
-      </c>
-      <c r="L13" s="10" t="n">
-        <v>5754.945</v>
-      </c>
-      <c r="M13" s="9" t="inlineStr">
-        <is>
-          <t>pending (time_all.sh not run yet)</t>
-        </is>
-      </c>
-      <c r="N13" s="17" t="n"/>
-      <c r="O13" s="11" t="inlineStr">
-        <is>
-          <t>nsys-20261015-091708.sqlite</t>
-        </is>
-      </c>
-      <c r="P13" s="18" t="n"/>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>pending (agentic optimized not profiled yet)</t>
-        </is>
-      </c>
-      <c r="R13" s="18" t="n"/>
-      <c r="S13" s="18" t="n"/>
-      <c r="T13" s="18" t="n"/>
-      <c r="U13" s="15" t="n">
-        <v>1.648</v>
-      </c>
-      <c r="V13" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!L13),ISNUMBER(L13)),'RTX 3090'!L13/L13,"pending")</f>
-        <v/>
-      </c>
-      <c r="W13" s="15" t="n"/>
-      <c r="X13" s="15" t="n"/>
-      <c r="Y13" s="5" t="inlineStr">
-        <is>
-          <t>Median GPU span of the 1693 graph replays with copies in the nsys traces. The CSR graph is uploaded from pinned memory in 8 chunks overlapped with the first iteration. A separate uninstrumented run of the binary (profiles/bench-20261015-091815.txt): 5.714 ms with transfers, 2.651 ms compute only.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny anomaly</t>
+          <t>pagerank (GAPBS)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>mse_partial_kernel</t>
+          <t>Whole application (H2D + 20 iterations + D2H)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>64M elements</t>
+          <t>2^20 vertices, 16 edges/vertex, 20 iterations</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -3045,89 +3669,75 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>Iteration time (nsys)</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="n"/>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
           <t>pending (direct mode not profiled yet)</t>
         </is>
       </c>
+      <c r="H15" s="16" t="n"/>
       <c r="I15" s="16" t="n"/>
       <c r="J15" s="16" t="n"/>
       <c r="K15" s="9" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="L15" s="10" t="n">
+        <v>5754.945</v>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>pending (ncu not run yet)</t>
+          <t>pending (time_all.sh not run yet)</t>
         </is>
       </c>
       <c r="N15" s="17" t="n"/>
       <c r="O15" s="11" t="inlineStr">
         <is>
-          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
-        </is>
-      </c>
-      <c r="P15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>nsys-20261015-091708.sqlite</t>
+        </is>
+      </c>
+      <c r="P15" s="18" t="n"/>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R15" s="12" t="inlineStr">
-        <is>
           <t>pending (agentic optimized not profiled yet)</t>
         </is>
       </c>
+      <c r="R15" s="18" t="n"/>
       <c r="S15" s="18" t="n"/>
       <c r="T15" s="18" t="n"/>
       <c r="U15" s="15" t="n">
-        <v>1.106</v>
+        <v>1.648</v>
       </c>
       <c r="V15" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!M15),ISNUMBER(M15)),'RTX 3090'!M15/M15,"pending")</f>
+        <f>IF(AND(ISNUMBER('RTX 3090'!L15),ISNUMBER(L15)),'RTX 3090'!L15/L15,"pending")</f>
         <v/>
       </c>
       <c r="W15" s="15" t="n"/>
       <c r="X15" s="15" t="n"/>
-      <c r="Y15" s="5" t="inlineStr"/>
+      <c r="Y15" s="5" t="inlineStr">
+        <is>
+          <t>Median GPU span of the 1693 graph replays with copies in the nsys traces. The CSR graph is uploaded from pinned memory in 8 chunks overlapped with the first iteration. A separate uninstrumented run of the binary (profiles/bench-20261015-091815.txt): 5.714 ms with transfers, 2.651 ms compute only.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny anomaly</t>
+          <t>pagerank (GAPBS)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Whole application (H2D + kernels + D2H)</t>
+          <t>Whole application, small shape (launch-bound)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>64M elements</t>
+          <t>2^14 vertices, 16 edges/vertex, 20 iterations</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -3137,49 +3747,37 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Iteration time (nsys)</t>
+          <t>Batch and single iteration (cudaEvent)</t>
         </is>
       </c>
       <c r="F16" s="16" t="n"/>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>pending (direct mode not profiled yet)</t>
+          <t>pending (time_all.sh not run yet)</t>
         </is>
       </c>
       <c r="H16" s="16" t="n"/>
       <c r="I16" s="16" t="n"/>
       <c r="J16" s="16" t="n"/>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>pending (time_all.sh not run yet)</t>
         </is>
       </c>
-      <c r="L16" s="10" t="n">
-        <v>13698.465</v>
-      </c>
-      <c r="M16" s="9" t="inlineStr">
-        <is>
-          <t>pending (time_all.sh not run yet)</t>
-        </is>
-      </c>
+      <c r="M16" s="17" t="n"/>
       <c r="N16" s="17" t="n"/>
-      <c r="O16" s="11" t="inlineStr">
-        <is>
-          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
-        </is>
-      </c>
+      <c r="O16" s="17" t="n"/>
       <c r="P16" s="18" t="n"/>
       <c r="Q16" s="12" t="inlineStr">
         <is>
-          <t>pending (agentic optimized not profiled yet)</t>
+          <t>pending (time_all.sh not run yet)</t>
         </is>
       </c>
       <c r="R16" s="18" t="n"/>
       <c r="S16" s="18" t="n"/>
       <c r="T16" s="18" t="n"/>
-      <c r="U16" s="15" t="n">
-        <v>1.003</v>
-      </c>
+      <c r="U16" s="15" t="n"/>
       <c r="V16" s="15">
         <f>IF(AND(ISNUMBER('RTX 3090'!L16),ISNUMBER(L16)),'RTX 3090'!L16/L16,"pending")</f>
         <v/>
@@ -3188,24 +3786,24 @@
       <c r="X16" s="15" t="n"/>
       <c r="Y16" s="5" t="inlineStr">
         <is>
-          <t>Median GPU span of the 41 graph replays with copies in the nsys traces.</t>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The same PageRank run on a 2^14-vertex graph (make -C pagerank small): upload, 20 iterations of a few microseconds each, download.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny KWS</t>
+          <t>mlperf-tiny anomaly</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>kws_postprocess_kernel</t>
+          <t>mse_partial_kernel</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>12 classes x 4M rows</t>
+          <t>64M elements</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -3253,7 +3851,7 @@
       <c r="N18" s="17" t="n"/>
       <c r="O18" s="11" t="inlineStr">
         <is>
-          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
         </is>
       </c>
       <c r="P18" s="12" t="inlineStr">
@@ -3274,7 +3872,7 @@
       <c r="S18" s="18" t="n"/>
       <c r="T18" s="18" t="n"/>
       <c r="U18" s="15" t="n">
-        <v>2.325</v>
+        <v>1.106</v>
       </c>
       <c r="V18" s="15">
         <f>IF(AND(ISNUMBER('RTX 3090'!M18),ISNUMBER(M18)),'RTX 3090'!M18/M18,"pending")</f>
@@ -3282,16 +3880,12 @@
       </c>
       <c r="W18" s="15" t="n"/>
       <c r="X18" s="15" t="n"/>
-      <c r="Y18" s="5" t="inlineStr">
-        <is>
-          <t>Only kernel in the application.</t>
-        </is>
-      </c>
+      <c r="Y18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny KWS</t>
+          <t>mlperf-tiny anomaly</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -3301,7 +3895,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>12 classes x 4M rows</t>
+          <t>64M elements</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -3329,7 +3923,7 @@
         </is>
       </c>
       <c r="L19" s="10" t="n">
-        <v>11226.082</v>
+        <v>13698.465</v>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
@@ -3339,7 +3933,7 @@
       <c r="N19" s="17" t="n"/>
       <c r="O19" s="11" t="inlineStr">
         <is>
-          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+          <t>nsys-anomaly_mse-20261015-091800.sqlite</t>
         </is>
       </c>
       <c r="P19" s="18" t="n"/>
@@ -3352,7 +3946,7 @@
       <c r="S19" s="18" t="n"/>
       <c r="T19" s="18" t="n"/>
       <c r="U19" s="15" t="n">
-        <v>1.059</v>
+        <v>1.003</v>
       </c>
       <c r="V19" s="15">
         <f>IF(AND(ISNUMBER('RTX 3090'!L19),ISNUMBER(L19)),'RTX 3090'!L19/L19,"pending")</f>
@@ -3366,116 +3960,86 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>mlperf-tiny VWW</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>vww_preprocess_kernel</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>256M bytes</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny anomaly</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>16 elements (smoke)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>RTX 4090 (sm_89, 24 GB)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Kernel time (ncu, one launch)</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>pending (direct mode not profiled yet)</t>
-        </is>
-      </c>
-      <c r="I21" s="16" t="n"/>
-      <c r="J21" s="16" t="n"/>
-      <c r="K21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M21" s="9" t="inlineStr">
-        <is>
-          <t>pending (ncu not run yet)</t>
-        </is>
-      </c>
-      <c r="N21" s="17" t="n"/>
-      <c r="O21" s="11" t="inlineStr">
-        <is>
-          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
-        </is>
-      </c>
-      <c r="P21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="Q21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R21" s="12" t="inlineStr">
-        <is>
-          <t>pending (agentic optimized not profiled yet)</t>
-        </is>
-      </c>
-      <c r="S21" s="18" t="n"/>
-      <c r="T21" s="18" t="n"/>
-      <c r="U21" s="15" t="n">
-        <v>1.106</v>
-      </c>
-      <c r="V21" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!M21),ISNUMBER(M21)),'RTX 3090'!M21/M21,"pending")</f>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="17" t="n"/>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="n"/>
+      <c r="N20" s="17" t="n"/>
+      <c r="O20" s="17" t="n"/>
+      <c r="P20" s="18" t="n"/>
+      <c r="Q20" s="12" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="R20" s="18" t="n"/>
+      <c r="S20" s="18" t="n"/>
+      <c r="T20" s="18" t="n"/>
+      <c r="U20" s="15" t="n"/>
+      <c r="V20" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L20),ISNUMBER(L20)),'RTX 3090'!L20/L20,"pending")</f>
         <v/>
       </c>
-      <c r="W21" s="15" t="n"/>
-      <c r="X21" s="15" t="n"/>
-      <c r="Y21" s="5" t="inlineStr">
-        <is>
-          <t>Only kernel in the application.</t>
+      <c r="W20" s="15" t="n"/>
+      <c r="X20" s="15" t="n"/>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>mlperf-tiny VWW</t>
+          <t>mlperf-tiny KWS</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Whole application (H2D + kernels + D2H)</t>
+          <t>kws_postprocess_kernel</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>256M bytes</t>
+          <t>12 classes x 4M rows</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -3485,91 +4049,493 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Iteration time (nsys)</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="n"/>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
           <t>pending (direct mode not profiled yet)</t>
         </is>
       </c>
-      <c r="H22" s="16" t="n"/>
       <c r="I22" s="16" t="n"/>
       <c r="J22" s="16" t="n"/>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>pending (time_all.sh not run yet)</t>
-        </is>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>21789.123</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>pending (time_all.sh not run yet)</t>
+          <t>pending (ncu not run yet)</t>
         </is>
       </c>
       <c r="N22" s="17" t="n"/>
       <c r="O22" s="11" t="inlineStr">
         <is>
-          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
-        </is>
-      </c>
-      <c r="P22" s="18" t="n"/>
+          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+        </is>
+      </c>
+      <c r="P22" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="Q22" s="12" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R22" s="12" t="inlineStr">
+        <is>
           <t>pending (agentic optimized not profiled yet)</t>
         </is>
       </c>
-      <c r="R22" s="18" t="n"/>
       <c r="S22" s="18" t="n"/>
       <c r="T22" s="18" t="n"/>
       <c r="U22" s="15" t="n">
-        <v>1.003</v>
+        <v>2.325</v>
       </c>
       <c r="V22" s="15">
-        <f>IF(AND(ISNUMBER('RTX 3090'!L22),ISNUMBER(L22)),'RTX 3090'!L22/L22,"pending")</f>
+        <f>IF(AND(ISNUMBER('RTX 3090'!M22),ISNUMBER(M22)),'RTX 3090'!M22/M22,"pending")</f>
         <v/>
       </c>
       <c r="W22" s="15" t="n"/>
       <c r="X22" s="15" t="n"/>
       <c r="Y22" s="5" t="inlineStr">
         <is>
+          <t>Only kernel in the application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 4M rows</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Iteration time (nsys)</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="n"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>pending (direct mode not profiled yet)</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="n"/>
+      <c r="I23" s="16" t="n"/>
+      <c r="J23" s="16" t="n"/>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>11226.082</v>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="n"/>
+      <c r="O23" s="11" t="inlineStr">
+        <is>
+          <t>nsys-kws_postprocess-20261015-091805.sqlite</t>
+        </is>
+      </c>
+      <c r="P23" s="18" t="n"/>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>pending (agentic optimized not profiled yet)</t>
+        </is>
+      </c>
+      <c r="R23" s="18" t="n"/>
+      <c r="S23" s="18" t="n"/>
+      <c r="T23" s="18" t="n"/>
+      <c r="U23" s="15" t="n">
+        <v>1.059</v>
+      </c>
+      <c r="V23" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L23),ISNUMBER(L23)),'RTX 3090'!L23/L23,"pending")</f>
+        <v/>
+      </c>
+      <c r="W23" s="15" t="n"/>
+      <c r="X23" s="15" t="n"/>
+      <c r="Y23" s="5" t="inlineStr">
+        <is>
           <t>Median GPU span of the 41 graph replays with copies in the nsys traces.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny KWS</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>12 classes x 1 row (smoke)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="n"/>
+      <c r="I24" s="16" t="n"/>
+      <c r="J24" s="16" t="n"/>
+      <c r="K24" s="17" t="n"/>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="M24" s="17" t="n"/>
+      <c r="N24" s="17" t="n"/>
+      <c r="O24" s="17" t="n"/>
+      <c r="P24" s="18" t="n"/>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="R24" s="18" t="n"/>
+      <c r="S24" s="18" t="n"/>
+      <c r="T24" s="18" t="n"/>
+      <c r="U24" s="15" t="n"/>
+      <c r="V24" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L24),ISNUMBER(L24)),'RTX 3090'!L24/L24,"pending")</f>
+        <v/>
+      </c>
+      <c r="W24" s="15" t="n"/>
+      <c r="X24" s="15" t="n"/>
+      <c r="Y24" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>vww_preprocess_kernel</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Kernel time (ncu, one launch)</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>pending (direct mode not profiled yet)</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="n"/>
+      <c r="J26" s="16" t="n"/>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>pending (ncu not run yet)</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="n"/>
+      <c r="O26" s="11" t="inlineStr">
+        <is>
+          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q26" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R26" s="12" t="inlineStr">
+        <is>
+          <t>pending (agentic optimized not profiled yet)</t>
+        </is>
+      </c>
+      <c r="S26" s="18" t="n"/>
+      <c r="T26" s="18" t="n"/>
+      <c r="U26" s="15" t="n">
+        <v>1.106</v>
+      </c>
+      <c r="V26" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!M26),ISNUMBER(M26)),'RTX 3090'!M26/M26,"pending")</f>
+        <v/>
+      </c>
+      <c r="W26" s="15" t="n"/>
+      <c r="X26" s="15" t="n"/>
+      <c r="Y26" s="5" t="inlineStr">
+        <is>
+          <t>Only kernel in the application.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Whole application (H2D + kernels + D2H)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>256M bytes</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Iteration time (nsys)</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="n"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>pending (direct mode not profiled yet)</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="n"/>
+      <c r="I27" s="16" t="n"/>
+      <c r="J27" s="16" t="n"/>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="L27" s="10" t="n">
+        <v>21789.123</v>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="N27" s="17" t="n"/>
+      <c r="O27" s="11" t="inlineStr">
+        <is>
+          <t>nsys-vww_preprocess-20261015-091810.sqlite</t>
+        </is>
+      </c>
+      <c r="P27" s="18" t="n"/>
+      <c r="Q27" s="12" t="inlineStr">
+        <is>
+          <t>pending (agentic optimized not profiled yet)</t>
+        </is>
+      </c>
+      <c r="R27" s="18" t="n"/>
+      <c r="S27" s="18" t="n"/>
+      <c r="T27" s="18" t="n"/>
+      <c r="U27" s="15" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="V27" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L27),ISNUMBER(L27)),'RTX 3090'!L27/L27,"pending")</f>
+        <v/>
+      </c>
+      <c r="W27" s="15" t="n"/>
+      <c r="X27" s="15" t="n"/>
+      <c r="Y27" s="5" t="inlineStr">
+        <is>
+          <t>Median GPU span of the 41 graph replays with copies in the nsys traces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>mlperf-tiny VWW</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Whole application, small shape (launch-bound)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>16 bytes (smoke)</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>RTX 4090 (sm_89, 24 GB)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Batch and single iteration (cudaEvent)</t>
+        </is>
+      </c>
+      <c r="F28" s="16" t="n"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="n"/>
+      <c r="I28" s="16" t="n"/>
+      <c r="J28" s="16" t="n"/>
+      <c r="K28" s="17" t="n"/>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="M28" s="17" t="n"/>
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="17" t="n"/>
+      <c r="P28" s="18" t="n"/>
+      <c r="Q28" s="12" t="inlineStr">
+        <is>
+          <t>pending (time_all.sh not run yet)</t>
+        </is>
+      </c>
+      <c r="R28" s="18" t="n"/>
+      <c r="S28" s="18" t="n"/>
+      <c r="T28" s="18" t="n"/>
+      <c r="U28" s="15" t="n"/>
+      <c r="V28" s="15">
+        <f>IF(AND(ISNUMBER('RTX 3090'!L28),ISNUMBER(L28)),'RTX 3090'!L28/L28,"pending")</f>
+        <v/>
+      </c>
+      <c r="W28" s="15" t="n"/>
+      <c r="X28" s="15" t="n"/>
+      <c r="Y28" s="5" t="inlineStr">
+        <is>
+          <t>Small shape, so launch cost dominates: compare the Graph speedup and Single / batch columns with the large-shape row above. A Single / batch below 1x means back-to-back iterations run slower than one alone, i.e. the batch is limited by how fast the host enqueues iterations rather than by the GPU. The smoke size on random inputs, including the H2D and D2H copies of a few bytes each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>How the predicted speedup is calculated (hover a Predicted value for that row's reason)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="31" ht="48" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
         <is>
           <t>The predicted speedup uses only the RTX 3090's ncu reports and the two GPUs' published specs (RTX 3090: 82 SMs, 1.695 GHz boost, 19.5 Gbps GDDR6X; RTX 4090: 128 SMs, 2.52 GHz boost, 21 Gbps GDDR6X; both 384-bit, PCIe 4.0 x16), so it is fixed before any 4090 measurement. Each unit's peak scales by its hardware ratio: SM compute by SMs x SM clock, L1/L2 cache throughput assumed to scale the same way, DRAM by memory data rate (the 3090's own SM and memory clocks come from its ncu report: 1.69 GHz and 18.98 Gbps, so the ratios are about 2.32x and 1.11x).</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>Kernel rows: ncu gives each launch's SM, memory (L1/L2) and DRAM throughput as a percent of the 3090's peak. Keeping the work per unit fixed, a unit at u% that is r times faster needs u/r% of the old time, and the slowest unit sets the new time: speedup = max(u) / max(u / r). So a DRAM-bound kernel gets ~1.11x and a compute- or cache-bound one ~2.32x. A launch below 60% on every unit is latency-bound and gets the SM clock ratio (1.49x). A kernel with several launches combines them weighted by time.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="48" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>Whole-application rows: the kernels in that workload's ncu report (one run of the application) scale by their predicted speedups; the rest of the 3090 time (H2D/D2H copies over the same PCIe 4.0 link, launch gaps) is assumed unchanged. Where the kernels overlap (llama2c's three streams; their summed time exceeds the iteration time), the whole time scales with the kernels.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1">
-      <c r="A28" s="20" t="inlineStr">
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>Not modelled: cache capacity (the 4090's L2 is 72 MB vs 6 MB, so data that spilled to DRAM on the 3090 can stay in L2), kernels overlapping copies (pagerank's first iteration), clocks above rated boost, and compiler differences (CUDA 13.3 vs 12.5). Measured = 3090 time / 4090 time for the CUDA Graph column; kernel rows read pending until the 4090 ncu reports exist.</t>
         </is>
@@ -3578,18 +4544,18 @@
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="W4:X4"/>
-    <mergeCell ref="A25:Y25"/>
     <mergeCell ref="A2:Y2"/>
     <mergeCell ref="P4:T4"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A28:Y28"/>
+    <mergeCell ref="A33:Y33"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A32:Y32"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="Y4:Y5"/>
-    <mergeCell ref="A27:Y27"/>
-    <mergeCell ref="A26:Y26"/>
+    <mergeCell ref="A31:Y31"/>
+    <mergeCell ref="A34:Y34"/>
     <mergeCell ref="K4:O4"/>
     <mergeCell ref="F4:J4"/>
     <mergeCell ref="U4:V4"/>
@@ -3601,21 +4567,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>